<commit_message>
chore: refresh docs and harden file workflows
</commit_message>
<xml_diff>
--- a/docs/test/接口扁平化测试用例.xlsx
+++ b/docs/test/接口扁平化测试用例.xlsx
@@ -9,12 +9,12 @@
   <sheets>
     <sheet name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="接口参数列表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="执行结果(标准环境R7)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="执行结果(标准环境R11)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$M$135</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$M$136</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'接口参数列表'!$A$1:$K$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'执行结果(标准环境R7)'!$A$1:$G$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'执行结果(标准环境R11)'!$A$1:$G$78</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M135"/>
+  <dimension ref="A1:M136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2115,17 +2115,17 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>200→SUCCESS(0行)</t>
+          <t>400</t>
         </is>
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>提交返回 taskId；最终 status=SUCCESS、imported=0（文件被解析为 0 行）</t>
-        </is>
-      </c>
-      <c r="M26" s="9" t="inlineStr">
-        <is>
-          <t>⚠️F-12：非 Excel 文件未拦截，静默成功，建议加文件头校验</t>
+          <t>提交阶段校验 .xlsx 后缀、zip 文件头和 xlsx 必要结构；非法文件不创建异步任务</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>F-12 已修复</t>
         </is>
       </c>
     </row>
@@ -6052,7 +6052,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>FIL-IC-01</t>
+          <t>FIL-UP-04</t>
         </is>
       </c>
       <c r="B91" s="12" t="inlineStr">
@@ -6062,22 +6062,22 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>POST /api/files/instant-check</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>POST /api/files/upload</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>安全</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>已上传某文件得到 md5/size</t>
+          <t>伪装可执行文件</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -6087,35 +6087,35 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>/api/files/instant-check</t>
+          <t>/api/files/upload</t>
         </is>
       </c>
       <c r="I91" s="5" t="inlineStr"/>
       <c r="J91" s="5" t="inlineStr">
         <is>
-          <t>{"fileMd5":"&lt;32位md5&gt;","fileSize":123}</t>
+          <t>file=@evil.xlsx(MZ头)</t>
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="L91" s="5" t="inlineStr">
         <is>
-          <t>命中：exists=true 并返回 file 信息</t>
+          <t>文件安全扫描拦截，不落库不生成 NORMAL 文件</t>
         </is>
       </c>
       <c r="M91" s="5" t="inlineStr">
         <is>
-          <t>秒传命中</t>
+          <t>内容嗅探</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>FIL-IC-02</t>
+          <t>FIL-IC-01</t>
         </is>
       </c>
       <c r="B92" s="12" t="inlineStr">
@@ -6128,9 +6128,9 @@
           <t>POST /api/files/instant-check</t>
         </is>
       </c>
-      <c r="D92" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -6140,7 +6140,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>md5/size 未命中</t>
+          <t>已上传某文件得到 md5/size</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -6156,7 +6156,7 @@
       <c r="I92" s="5" t="inlineStr"/>
       <c r="J92" s="5" t="inlineStr">
         <is>
-          <t>{"fileMd5":"0000...0001","fileSize":123}</t>
+          <t>{"fileMd5":"&lt;32位md5&gt;","fileSize":123}</t>
         </is>
       </c>
       <c r="K92" s="2" t="inlineStr">
@@ -6166,19 +6166,19 @@
       </c>
       <c r="L92" s="5" t="inlineStr">
         <is>
-          <t>exists=false，file=null</t>
+          <t>命中：exists=true 并返回 file 信息</t>
         </is>
       </c>
       <c r="M92" s="5" t="inlineStr">
         <is>
-          <t>秒传未命中</t>
+          <t>秒传命中</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>FIL-IC-03</t>
+          <t>FIL-IC-02</t>
         </is>
       </c>
       <c r="B93" s="12" t="inlineStr">
@@ -6198,12 +6198,12 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>异常</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>md5/size 未命中</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -6219,25 +6219,29 @@
       <c r="I93" s="5" t="inlineStr"/>
       <c r="J93" s="5" t="inlineStr">
         <is>
-          <t>{"fileMd5":"","fileSize":123}</t>
+          <t>{"fileMd5":"0000...0001","fileSize":123}</t>
         </is>
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L93" s="5" t="inlineStr">
         <is>
-          <t>“文件 MD5 不能为空”</t>
-        </is>
-      </c>
-      <c r="M93" s="5" t="inlineStr"/>
+          <t>exists=false，file=null</t>
+        </is>
+      </c>
+      <c r="M93" s="5" t="inlineStr">
+        <is>
+          <t>秒传未命中</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>FIL-IC-04</t>
+          <t>FIL-IC-03</t>
         </is>
       </c>
       <c r="B94" s="12" t="inlineStr">
@@ -6250,14 +6254,14 @@
           <t>POST /api/files/instant-check</t>
         </is>
       </c>
-      <c r="D94" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D94" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>边界</t>
+          <t>异常</t>
         </is>
       </c>
       <c r="F94" s="5" t="inlineStr">
@@ -6278,7 +6282,7 @@
       <c r="I94" s="5" t="inlineStr"/>
       <c r="J94" s="5" t="inlineStr">
         <is>
-          <t>{"fileMd5":"not-hex","fileSize":123}</t>
+          <t>{"fileMd5":"","fileSize":123}</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr">
@@ -6288,7 +6292,7 @@
       </c>
       <c r="L94" s="5" t="inlineStr">
         <is>
-          <t>“文件 MD5 格式不正确”（需 32 位小写十六进制）</t>
+          <t>“文件 MD5 不能为空”</t>
         </is>
       </c>
       <c r="M94" s="5" t="inlineStr"/>
@@ -6296,7 +6300,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>FIL-IC-05</t>
+          <t>FIL-IC-04</t>
         </is>
       </c>
       <c r="B95" s="12" t="inlineStr">
@@ -6337,7 +6341,7 @@
       <c r="I95" s="5" t="inlineStr"/>
       <c r="J95" s="5" t="inlineStr">
         <is>
-          <t>{"fileMd5":"&lt;32位md5&gt;","fileSize":0}</t>
+          <t>{"fileMd5":"not-hex","fileSize":123}</t>
         </is>
       </c>
       <c r="K95" s="2" t="inlineStr">
@@ -6347,7 +6351,7 @@
       </c>
       <c r="L95" s="5" t="inlineStr">
         <is>
-          <t>“文件大小必须大于 0”</t>
+          <t>“文件 MD5 格式不正确”（需 32 位小写十六进制）</t>
         </is>
       </c>
       <c r="M95" s="5" t="inlineStr"/>
@@ -6355,7 +6359,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>FIL-DI-01</t>
+          <t>FIL-IC-05</t>
         </is>
       </c>
       <c r="B96" s="12" t="inlineStr">
@@ -6365,22 +6369,22 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>POST /api/files/direct/init</t>
-        </is>
-      </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>POST /api/files/instant-check</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>边界</t>
         </is>
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>md5 未命中</t>
+          <t>无</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -6390,23 +6394,23 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>/api/files/direct/init</t>
+          <t>/api/files/instant-check</t>
         </is>
       </c>
       <c r="I96" s="5" t="inlineStr"/>
       <c r="J96" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"demo.zip","contentType":"application/zip","fileSize":1024,"fileMd5":"&lt;32位&gt;"}</t>
+          <t>{"fileMd5":"&lt;32位md5&gt;","fileSize":0}</t>
         </is>
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="L96" s="5" t="inlineStr">
         <is>
-          <t>instant=false；返回 uploadId/fileId/uploadUrl/objectKey/expireMinutes</t>
+          <t>“文件大小必须大于 0”</t>
         </is>
       </c>
       <c r="M96" s="5" t="inlineStr"/>
@@ -6414,7 +6418,7 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>FIL-DI-02</t>
+          <t>FIL-DI-01</t>
         </is>
       </c>
       <c r="B97" s="12" t="inlineStr">
@@ -6427,9 +6431,9 @@
           <t>POST /api/files/direct/init</t>
         </is>
       </c>
-      <c r="D97" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -6439,7 +6443,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>md5 命中</t>
+          <t>md5 未命中</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -6455,7 +6459,7 @@
       <c r="I97" s="5" t="inlineStr"/>
       <c r="J97" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"demo.zip","fileSize":&lt;size&gt;,"fileMd5":"&lt;已存在md5&gt;"}</t>
+          <t>{"originalName":"demo.zip","contentType":"application/zip","fileSize":1024,"fileMd5":"&lt;32位&gt;"}</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
@@ -6465,7 +6469,7 @@
       </c>
       <c r="L97" s="5" t="inlineStr">
         <is>
-          <t>instant=true；返回 fileId/file，无需上传</t>
+          <t>instant=false；返回 uploadId/fileId/uploadUrl/objectKey/expireMinutes</t>
         </is>
       </c>
       <c r="M97" s="5" t="inlineStr"/>
@@ -6473,7 +6477,7 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>FIL-DI-03</t>
+          <t>FIL-DI-02</t>
         </is>
       </c>
       <c r="B98" s="12" t="inlineStr">
@@ -6486,19 +6490,19 @@
           <t>POST /api/files/direct/init</t>
         </is>
       </c>
-      <c r="D98" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>边界</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>md5 命中</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -6514,7 +6518,7 @@
       <c r="I98" s="5" t="inlineStr"/>
       <c r="J98" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"","fileSize":1024,"fileMd5":"&lt;32位&gt;"}</t>
+          <t>{"originalName":"demo.zip","fileSize":&lt;size&gt;,"fileMd5":"&lt;已存在md5&gt;"}</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr">
@@ -6524,7 +6528,7 @@
       </c>
       <c r="L98" s="5" t="inlineStr">
         <is>
-          <t>originalName 缺省归一化为 unknown</t>
+          <t>instant=true；返回 fileId/file，无需上传</t>
         </is>
       </c>
       <c r="M98" s="5" t="inlineStr"/>
@@ -6532,7 +6536,7 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>FIL-DI-04</t>
+          <t>FIL-DI-03</t>
         </is>
       </c>
       <c r="B99" s="12" t="inlineStr">
@@ -6545,14 +6549,14 @@
           <t>POST /api/files/direct/init</t>
         </is>
       </c>
-      <c r="D99" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>异常</t>
+          <t>边界</t>
         </is>
       </c>
       <c r="F99" s="5" t="inlineStr">
@@ -6573,17 +6577,17 @@
       <c r="I99" s="5" t="inlineStr"/>
       <c r="J99" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"x","fileSize":1024,"fileMd5":"bad"}</t>
+          <t>{"originalName":"","fileSize":1024,"fileMd5":"&lt;32位&gt;"}</t>
         </is>
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L99" s="5" t="inlineStr">
         <is>
-          <t>MD5 格式校验失败</t>
+          <t>originalName 缺省归一化为 unknown</t>
         </is>
       </c>
       <c r="M99" s="5" t="inlineStr"/>
@@ -6591,7 +6595,7 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>FIL-DI-05</t>
+          <t>FIL-DI-04</t>
         </is>
       </c>
       <c r="B100" s="12" t="inlineStr">
@@ -6604,14 +6608,14 @@
           <t>POST /api/files/direct/init</t>
         </is>
       </c>
-      <c r="D100" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>边界</t>
+          <t>异常</t>
         </is>
       </c>
       <c r="F100" s="5" t="inlineStr">
@@ -6632,7 +6636,7 @@
       <c r="I100" s="5" t="inlineStr"/>
       <c r="J100" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"x","fileSize":-1,"fileMd5":"&lt;32位&gt;"}</t>
+          <t>{"originalName":"x","fileSize":1024,"fileMd5":"bad"}</t>
         </is>
       </c>
       <c r="K100" s="2" t="inlineStr">
@@ -6642,7 +6646,7 @@
       </c>
       <c r="L100" s="5" t="inlineStr">
         <is>
-          <t>“文件大小必须大于 0”</t>
+          <t>MD5 格式校验失败</t>
         </is>
       </c>
       <c r="M100" s="5" t="inlineStr"/>
@@ -6650,7 +6654,7 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>FIL-DC-01</t>
+          <t>FIL-DI-05</t>
         </is>
       </c>
       <c r="B101" s="12" t="inlineStr">
@@ -6660,22 +6664,22 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>POST /api/files/direct/{uploadId}/complete</t>
-        </is>
-      </c>
-      <c r="D101" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>POST /api/files/direct/init</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>边界</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>已 init 并 PUT 完整对象到 MinIO</t>
+          <t>无</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -6685,19 +6689,23 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>/api/files/direct/{uploadId}/complete</t>
+          <t>/api/files/direct/init</t>
         </is>
       </c>
       <c r="I101" s="5" t="inlineStr"/>
-      <c r="J101" s="5" t="inlineStr"/>
+      <c r="J101" s="5" t="inlineStr">
+        <is>
+          <t>{"originalName":"x","fileSize":-1,"fileMd5":"&lt;32位&gt;"}</t>
+        </is>
+      </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="L101" s="5" t="inlineStr">
         <is>
-          <t>校验对象存在且大小匹配→生成 FileResponse，任务 SUCCESS</t>
+          <t>“文件大小必须大于 0”</t>
         </is>
       </c>
       <c r="M101" s="5" t="inlineStr"/>
@@ -6705,7 +6713,7 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>FIL-DC-02</t>
+          <t>FIL-DC-01</t>
         </is>
       </c>
       <c r="B102" s="12" t="inlineStr">
@@ -6725,12 +6733,12 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>异常</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>uploadId 不存在/类型不符</t>
+          <t>已 init 并 PUT 完整对象到 MinIO</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -6740,19 +6748,19 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>/api/files/direct/not-exist/complete</t>
+          <t>/api/files/direct/{uploadId}/complete</t>
         </is>
       </c>
       <c r="I102" s="5" t="inlineStr"/>
       <c r="J102" s="5" t="inlineStr"/>
       <c r="K102" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L102" s="5" t="inlineStr">
         <is>
-          <t>“上传任务不存在/类型不匹配”</t>
+          <t>校验对象存在且大小匹配→生成 FileResponse，任务 SUCCESS</t>
         </is>
       </c>
       <c r="M102" s="5" t="inlineStr"/>
@@ -6760,7 +6768,7 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>FIL-DC-03</t>
+          <t>FIL-DC-02</t>
         </is>
       </c>
       <c r="B103" s="12" t="inlineStr">
@@ -6780,12 +6788,12 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>业务规则</t>
+          <t>异常</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>任务非 UPLOADING（已完成/已取消）</t>
+          <t>uploadId 不存在/类型不符</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -6795,19 +6803,19 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>/api/files/direct/{uploadId}/complete</t>
+          <t>/api/files/direct/not-exist/complete</t>
         </is>
       </c>
       <c r="I103" s="5" t="inlineStr"/>
       <c r="J103" s="5" t="inlineStr"/>
       <c r="K103" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>404</t>
         </is>
       </c>
       <c r="L103" s="5" t="inlineStr">
         <is>
-          <t>“上传任务状态不允许完成”</t>
+          <t>“上传任务不存在/类型不匹配”</t>
         </is>
       </c>
       <c r="M103" s="5" t="inlineStr"/>
@@ -6815,7 +6823,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>FIL-DC-04</t>
+          <t>FIL-DC-03</t>
         </is>
       </c>
       <c r="B104" s="12" t="inlineStr">
@@ -6840,7 +6848,7 @@
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>对象大小与声明不符</t>
+          <t>任务非 UPLOADING（已完成/已取消）</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -6862,19 +6870,15 @@
       </c>
       <c r="L104" s="5" t="inlineStr">
         <is>
-          <t>“文件大小不匹配”</t>
-        </is>
-      </c>
-      <c r="M104" s="5" t="inlineStr">
-        <is>
-          <t>未 PUT 或内容错误</t>
-        </is>
-      </c>
+          <t>“上传任务状态不允许完成”</t>
+        </is>
+      </c>
+      <c r="M104" s="5" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>FIL-MI-01</t>
+          <t>FIL-DC-04</t>
         </is>
       </c>
       <c r="B105" s="12" t="inlineStr">
@@ -6884,22 +6888,22 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>POST /api/files/multipart/init</t>
-        </is>
-      </c>
-      <c r="D105" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>POST /api/files/direct/{uploadId}/complete</t>
+        </is>
+      </c>
+      <c r="D105" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>业务规则</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>大文件 md5 未命中</t>
+          <t>对象大小与声明不符</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -6909,31 +6913,31 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>/api/files/multipart/init</t>
+          <t>/api/files/direct/{uploadId}/complete</t>
         </is>
       </c>
       <c r="I105" s="5" t="inlineStr"/>
-      <c r="J105" s="5" t="inlineStr">
-        <is>
-          <t>{"originalName":"big.mp4","fileSize":16777216,"fileMd5":"&lt;32位&gt;","partSize":8388608}</t>
-        </is>
-      </c>
+      <c r="J105" s="5" t="inlineStr"/>
       <c r="K105" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>409</t>
         </is>
       </c>
       <c r="L105" s="5" t="inlineStr">
         <is>
-          <t>返回 uploadId/partCount(=2)/partSize/parts[每个含 uploadUrl、expectedSize]</t>
-        </is>
-      </c>
-      <c r="M105" s="5" t="inlineStr"/>
+          <t>“文件大小不匹配”</t>
+        </is>
+      </c>
+      <c r="M105" s="5" t="inlineStr">
+        <is>
+          <t>未 PUT 或内容错误</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>FIL-MI-02</t>
+          <t>FIL-MI-01</t>
         </is>
       </c>
       <c r="B106" s="12" t="inlineStr">
@@ -6946,19 +6950,19 @@
           <t>POST /api/files/multipart/init</t>
         </is>
       </c>
-      <c r="D106" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>边界</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
-          <t>partSize 小于 5MB</t>
+          <t>大文件 md5 未命中</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -6974,7 +6978,7 @@
       <c r="I106" s="5" t="inlineStr"/>
       <c r="J106" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"x","fileSize":16777216,"fileMd5":"&lt;32位&gt;","partSize":1048576}</t>
+          <t>{"originalName":"big.mp4","fileSize":16777216,"fileMd5":"&lt;32位&gt;","partSize":8388608}</t>
         </is>
       </c>
       <c r="K106" s="2" t="inlineStr">
@@ -6984,19 +6988,15 @@
       </c>
       <c r="L106" s="5" t="inlineStr">
         <is>
-          <t>partSize 被钳制为最小 5MB</t>
-        </is>
-      </c>
-      <c r="M106" s="5" t="inlineStr">
-        <is>
-          <t>最小分片 5MB</t>
-        </is>
-      </c>
+          <t>返回 uploadId/partCount(=2)/partSize/parts[每个含 uploadUrl、expectedSize]</t>
+        </is>
+      </c>
+      <c r="M106" s="5" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>FIL-MI-03</t>
+          <t>FIL-MI-02</t>
         </is>
       </c>
       <c r="B107" s="12" t="inlineStr">
@@ -7009,19 +7009,19 @@
           <t>POST /api/files/multipart/init</t>
         </is>
       </c>
-      <c r="D107" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="D107" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>业务规则</t>
+          <t>边界</t>
         </is>
       </c>
       <c r="F107" s="5" t="inlineStr">
         <is>
-          <t>分片数超过上限 1000</t>
+          <t>partSize 小于 5MB</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -7037,25 +7037,29 @@
       <c r="I107" s="5" t="inlineStr"/>
       <c r="J107" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"x","fileSize":100000000000,"fileMd5":"&lt;32位&gt;","partSize":8388608}</t>
+          <t>{"originalName":"x","fileSize":16777216,"fileMd5":"&lt;32位&gt;","partSize":1048576}</t>
         </is>
       </c>
       <c r="K107" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L107" s="5" t="inlineStr">
         <is>
-          <t>“文件分片数量超过上限”</t>
-        </is>
-      </c>
-      <c r="M107" s="5" t="inlineStr"/>
+          <t>partSize 被钳制为最小 5MB</t>
+        </is>
+      </c>
+      <c r="M107" s="5" t="inlineStr">
+        <is>
+          <t>最小分片 5MB</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>FIL-MI-04</t>
+          <t>FIL-MI-03</t>
         </is>
       </c>
       <c r="B108" s="12" t="inlineStr">
@@ -7075,12 +7079,12 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>业务规则</t>
         </is>
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>md5 命中秒传</t>
+          <t>分片数超过上限 1000</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -7096,17 +7100,17 @@
       <c r="I108" s="5" t="inlineStr"/>
       <c r="J108" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"x","fileSize":&lt;size&gt;,"fileMd5":"&lt;已存在&gt;"}</t>
+          <t>{"originalName":"x","fileSize":100000000000,"fileMd5":"&lt;32位&gt;","partSize":8388608}</t>
         </is>
       </c>
       <c r="K108" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="L108" s="5" t="inlineStr">
         <is>
-          <t>instant=true，不创建上传任务</t>
+          <t>“文件分片数量超过上限”</t>
         </is>
       </c>
       <c r="M108" s="5" t="inlineStr"/>
@@ -7114,7 +7118,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>FIL-MI-05</t>
+          <t>FIL-MI-04</t>
         </is>
       </c>
       <c r="B109" s="12" t="inlineStr">
@@ -7134,12 +7138,12 @@
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>异常</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>md5 命中秒传</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -7155,17 +7159,17 @@
       <c r="I109" s="5" t="inlineStr"/>
       <c r="J109" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"x","fileSize":1024,"fileMd5":"bad"}</t>
+          <t>{"originalName":"x","fileSize":&lt;size&gt;,"fileMd5":"&lt;已存在&gt;"}</t>
         </is>
       </c>
       <c r="K109" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L109" s="5" t="inlineStr">
         <is>
-          <t>MD5 格式校验失败</t>
+          <t>instant=true，不创建上传任务</t>
         </is>
       </c>
       <c r="M109" s="5" t="inlineStr"/>
@@ -7173,7 +7177,7 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>FIL-MI-06</t>
+          <t>FIL-MI-05</t>
         </is>
       </c>
       <c r="B110" s="12" t="inlineStr">
@@ -7186,19 +7190,19 @@
           <t>POST /api/files/multipart/init</t>
         </is>
       </c>
-      <c r="D110" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>边界</t>
+          <t>异常</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>单分片文件</t>
+          <t>无</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -7214,29 +7218,25 @@
       <c r="I110" s="5" t="inlineStr"/>
       <c r="J110" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"x","fileSize":1024,"fileMd5":"&lt;32位&gt;","partSize":8388608}</t>
+          <t>{"originalName":"x","fileSize":1024,"fileMd5":"bad"}</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="L110" s="5" t="inlineStr">
         <is>
-          <t>partCount=1</t>
-        </is>
-      </c>
-      <c r="M110" s="5" t="inlineStr">
-        <is>
-          <t>最小分片场景</t>
-        </is>
-      </c>
+          <t>MD5 格式校验失败</t>
+        </is>
+      </c>
+      <c r="M110" s="5" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>FIL-MP-01</t>
+          <t>FIL-MI-06</t>
         </is>
       </c>
       <c r="B111" s="12" t="inlineStr">
@@ -7246,36 +7246,40 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>GET /api/files/multipart/{uploadId}/parts</t>
-        </is>
-      </c>
-      <c r="D111" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>POST /api/files/multipart/init</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>边界</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>已 init 并上传部分分片</t>
+          <t>单分片文件</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>/api/files/multipart/{uploadId}/parts</t>
+          <t>/api/files/multipart/init</t>
         </is>
       </c>
       <c r="I111" s="5" t="inlineStr"/>
-      <c r="J111" s="5" t="inlineStr"/>
+      <c r="J111" s="5" t="inlineStr">
+        <is>
+          <t>{"originalName":"x","fileSize":1024,"fileMd5":"&lt;32位&gt;","partSize":8388608}</t>
+        </is>
+      </c>
       <c r="K111" s="2" t="inlineStr">
         <is>
           <t>200</t>
@@ -7283,19 +7287,19 @@
       </c>
       <c r="L111" s="5" t="inlineStr">
         <is>
-          <t>返回 partCount 与 uploadedParts（已上传分片序号）</t>
+          <t>partCount=1</t>
         </is>
       </c>
       <c r="M111" s="5" t="inlineStr">
         <is>
-          <t>断点续传依据</t>
+          <t>最小分片场景</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>FIL-MP-02</t>
+          <t>FIL-MP-01</t>
         </is>
       </c>
       <c r="B112" s="12" t="inlineStr">
@@ -7308,9 +7312,9 @@
           <t>GET /api/files/multipart/{uploadId}/parts</t>
         </is>
       </c>
-      <c r="D112" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -7320,7 +7324,7 @@
       </c>
       <c r="F112" s="5" t="inlineStr">
         <is>
-          <t>未上传任何分片</t>
+          <t>已 init 并上传部分分片</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -7342,15 +7346,19 @@
       </c>
       <c r="L112" s="5" t="inlineStr">
         <is>
-          <t>uploadedParts 为空数组</t>
-        </is>
-      </c>
-      <c r="M112" s="5" t="inlineStr"/>
+          <t>返回 partCount 与 uploadedParts（已上传分片序号）</t>
+        </is>
+      </c>
+      <c r="M112" s="5" t="inlineStr">
+        <is>
+          <t>断点续传依据</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>FIL-MP-03</t>
+          <t>FIL-MP-02</t>
         </is>
       </c>
       <c r="B113" s="12" t="inlineStr">
@@ -7363,19 +7371,19 @@
           <t>GET /api/files/multipart/{uploadId}/parts</t>
         </is>
       </c>
-      <c r="D113" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="D113" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>异常</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
-          <t>uploadId 不存在/类型不符</t>
+          <t>未上传任何分片</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -7385,19 +7393,19 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>/api/files/multipart/not-exist/parts</t>
+          <t>/api/files/multipart/{uploadId}/parts</t>
         </is>
       </c>
       <c r="I113" s="5" t="inlineStr"/>
       <c r="J113" s="5" t="inlineStr"/>
       <c r="K113" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L113" s="5" t="inlineStr">
         <is>
-          <t>“上传任务不存在/类型不匹配”</t>
+          <t>uploadedParts 为空数组</t>
         </is>
       </c>
       <c r="M113" s="5" t="inlineStr"/>
@@ -7405,7 +7413,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>FIL-MC-01</t>
+          <t>FIL-MP-03</t>
         </is>
       </c>
       <c r="B114" s="12" t="inlineStr">
@@ -7415,7 +7423,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>POST /api/files/multipart/{uploadId}/complete</t>
+          <t>GET /api/files/multipart/{uploadId}/parts</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
@@ -7425,34 +7433,34 @@
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>异常</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
         <is>
-          <t>全部分片已 PUT</t>
+          <t>uploadId 不存在/类型不符</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>/api/files/multipart/{uploadId}/complete</t>
+          <t>/api/files/multipart/not-exist/parts</t>
         </is>
       </c>
       <c r="I114" s="5" t="inlineStr"/>
       <c r="J114" s="5" t="inlineStr"/>
       <c r="K114" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="L114" s="5" t="inlineStr">
         <is>
-          <t>逐片校验→composeObject→生成 FileResponse，任务 SUCCESS</t>
+          <t>“上传任务不存在/类型不匹配”</t>
         </is>
       </c>
       <c r="M114" s="5" t="inlineStr"/>
@@ -7460,7 +7468,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>FIL-MC-02</t>
+          <t>FIL-MC-01</t>
         </is>
       </c>
       <c r="B115" s="12" t="inlineStr">
@@ -7480,12 +7488,12 @@
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>业务规则</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F115" s="5" t="inlineStr">
         <is>
-          <t>缺少分片</t>
+          <t>全部分片已 PUT</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -7502,12 +7510,12 @@
       <c r="J115" s="5" t="inlineStr"/>
       <c r="K115" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L115" s="5" t="inlineStr">
         <is>
-          <t>分片对象不存在/大小为 0，抛 IllegalStateException</t>
+          <t>逐片校验→composeObject→生成 FileResponse，任务 SUCCESS</t>
         </is>
       </c>
       <c r="M115" s="5" t="inlineStr"/>
@@ -7515,7 +7523,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>FIL-MC-03</t>
+          <t>FIL-MC-02</t>
         </is>
       </c>
       <c r="B116" s="12" t="inlineStr">
@@ -7540,7 +7548,7 @@
       </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
-          <t>某分片大小与 expected 不符</t>
+          <t>缺少分片</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -7562,7 +7570,7 @@
       </c>
       <c r="L116" s="5" t="inlineStr">
         <is>
-          <t>“分片大小不匹配”</t>
+          <t>分片对象不存在/大小为 0，抛 IllegalStateException</t>
         </is>
       </c>
       <c r="M116" s="5" t="inlineStr"/>
@@ -7570,7 +7578,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>FIL-MC-04</t>
+          <t>FIL-MC-03</t>
         </is>
       </c>
       <c r="B117" s="12" t="inlineStr">
@@ -7583,9 +7591,9 @@
           <t>POST /api/files/multipart/{uploadId}/complete</t>
         </is>
       </c>
-      <c r="D117" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
@@ -7595,7 +7603,7 @@
       </c>
       <c r="F117" s="5" t="inlineStr">
         <is>
-          <t>合并对象总大小与声明不符</t>
+          <t>某分片大小与 expected 不符</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -7617,7 +7625,7 @@
       </c>
       <c r="L117" s="5" t="inlineStr">
         <is>
-          <t>“文件大小不匹配”</t>
+          <t>“分片大小不匹配”</t>
         </is>
       </c>
       <c r="M117" s="5" t="inlineStr"/>
@@ -7625,7 +7633,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>FIL-MC-05</t>
+          <t>FIL-MC-04</t>
         </is>
       </c>
       <c r="B118" s="12" t="inlineStr">
@@ -7638,9 +7646,9 @@
           <t>POST /api/files/multipart/{uploadId}/complete</t>
         </is>
       </c>
-      <c r="D118" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="D118" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -7650,7 +7658,7 @@
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
-          <t>任务非 UPLOADING</t>
+          <t>合并对象总大小与声明不符</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -7672,7 +7680,7 @@
       </c>
       <c r="L118" s="5" t="inlineStr">
         <is>
-          <t>“上传任务状态不允许完成”</t>
+          <t>“文件大小不匹配”</t>
         </is>
       </c>
       <c r="M118" s="5" t="inlineStr"/>
@@ -7680,7 +7688,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>FIL-MC-06</t>
+          <t>FIL-MC-05</t>
         </is>
       </c>
       <c r="B119" s="12" t="inlineStr">
@@ -7700,12 +7708,12 @@
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>异常</t>
+          <t>业务规则</t>
         </is>
       </c>
       <c r="F119" s="5" t="inlineStr">
         <is>
-          <t>uploadId 不存在</t>
+          <t>任务非 UPLOADING</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -7715,19 +7723,19 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>/api/files/multipart/not-exist/complete</t>
+          <t>/api/files/multipart/{uploadId}/complete</t>
         </is>
       </c>
       <c r="I119" s="5" t="inlineStr"/>
       <c r="J119" s="5" t="inlineStr"/>
       <c r="K119" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>409</t>
         </is>
       </c>
       <c r="L119" s="5" t="inlineStr">
         <is>
-          <t>“上传任务不存在”</t>
+          <t>“上传任务状态不允许完成”</t>
         </is>
       </c>
       <c r="M119" s="5" t="inlineStr"/>
@@ -7735,7 +7743,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>FIL-MA-01</t>
+          <t>FIL-MC-06</t>
         </is>
       </c>
       <c r="B120" s="12" t="inlineStr">
@@ -7745,7 +7753,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>POST /api/files/multipart/{uploadId}/abort</t>
+          <t>POST /api/files/multipart/{uploadId}/complete</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
@@ -7755,12 +7763,12 @@
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>异常</t>
         </is>
       </c>
       <c r="F120" s="5" t="inlineStr">
         <is>
-          <t>已 init 的分片任务</t>
+          <t>uploadId 不存在</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -7770,19 +7778,19 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>/api/files/multipart/{uploadId}/abort</t>
+          <t>/api/files/multipart/not-exist/complete</t>
         </is>
       </c>
       <c r="I120" s="5" t="inlineStr"/>
       <c r="J120" s="5" t="inlineStr"/>
       <c r="K120" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="L120" s="5" t="inlineStr">
         <is>
-          <t>aborted=true；任务 ABORTED，提交后清理临时分片</t>
+          <t>“上传任务不存在”</t>
         </is>
       </c>
       <c r="M120" s="5" t="inlineStr"/>
@@ -7790,7 +7798,7 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>FIL-MA-02</t>
+          <t>FIL-MA-01</t>
         </is>
       </c>
       <c r="B121" s="12" t="inlineStr">
@@ -7803,19 +7811,19 @@
           <t>POST /api/files/multipart/{uploadId}/abort</t>
         </is>
       </c>
-      <c r="D121" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>业务规则</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F121" s="5" t="inlineStr">
         <is>
-          <t>任务已 ABORTED/SUCCESS</t>
+          <t>已 init 的分片任务</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -7832,12 +7840,12 @@
       <c r="J121" s="5" t="inlineStr"/>
       <c r="K121" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L121" s="5" t="inlineStr">
         <is>
-          <t>非 UPLOADING 抛 IllegalStateException</t>
+          <t>aborted=true；任务 ABORTED，提交后清理临时分片</t>
         </is>
       </c>
       <c r="M121" s="5" t="inlineStr"/>
@@ -7845,7 +7853,7 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>FIL-MA-03</t>
+          <t>FIL-MA-02</t>
         </is>
       </c>
       <c r="B122" s="12" t="inlineStr">
@@ -7858,19 +7866,19 @@
           <t>POST /api/files/multipart/{uploadId}/abort</t>
         </is>
       </c>
-      <c r="D122" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="D122" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>异常</t>
+          <t>业务规则</t>
         </is>
       </c>
       <c r="F122" s="5" t="inlineStr">
         <is>
-          <t>uploadId 不存在</t>
+          <t>任务已 ABORTED/SUCCESS</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -7880,19 +7888,19 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>/api/files/multipart/not-exist/abort</t>
+          <t>/api/files/multipart/{uploadId}/abort</t>
         </is>
       </c>
       <c r="I122" s="5" t="inlineStr"/>
       <c r="J122" s="5" t="inlineStr"/>
       <c r="K122" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>409</t>
         </is>
       </c>
       <c r="L122" s="5" t="inlineStr">
         <is>
-          <t>“上传任务不存在”</t>
+          <t>非 UPLOADING 抛 IllegalStateException</t>
         </is>
       </c>
       <c r="M122" s="5" t="inlineStr"/>
@@ -7900,7 +7908,7 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>FIL-GET-01</t>
+          <t>FIL-MA-03</t>
         </is>
       </c>
       <c r="B123" s="12" t="inlineStr">
@@ -7910,44 +7918,44 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>GET /api/files/{fileId}</t>
-        </is>
-      </c>
-      <c r="D123" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>POST /api/files/multipart/{uploadId}/abort</t>
+        </is>
+      </c>
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>异常</t>
         </is>
       </c>
       <c r="F123" s="5" t="inlineStr">
         <is>
-          <t>存在 NORMAL 文件</t>
+          <t>uploadId 不存在</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>/api/files/{fileId}</t>
+          <t>/api/files/multipart/not-exist/abort</t>
         </is>
       </c>
       <c r="I123" s="5" t="inlineStr"/>
       <c r="J123" s="5" t="inlineStr"/>
       <c r="K123" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="L123" s="5" t="inlineStr">
         <is>
-          <t>返回 FileResponse（originalName/fileSize/fileMd5/fileExt/contentType/createdAt）</t>
+          <t>“上传任务不存在”</t>
         </is>
       </c>
       <c r="M123" s="5" t="inlineStr"/>
@@ -7955,7 +7963,7 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>FIL-GET-02</t>
+          <t>FIL-GET-01</t>
         </is>
       </c>
       <c r="B124" s="12" t="inlineStr">
@@ -7968,19 +7976,19 @@
           <t>GET /api/files/{fileId}</t>
         </is>
       </c>
-      <c r="D124" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>异常</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F124" s="5" t="inlineStr">
         <is>
-          <t>fileId 不存在</t>
+          <t>存在 NORMAL 文件</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -7990,19 +7998,19 @@
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>/api/files/not-exist</t>
+          <t>/api/files/{fileId}</t>
         </is>
       </c>
       <c r="I124" s="5" t="inlineStr"/>
       <c r="J124" s="5" t="inlineStr"/>
       <c r="K124" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L124" s="5" t="inlineStr">
         <is>
-          <t>“文件不存在”</t>
+          <t>返回 FileResponse（originalName/fileSize/fileMd5/fileExt/contentType/createdAt）</t>
         </is>
       </c>
       <c r="M124" s="5" t="inlineStr"/>
@@ -8010,7 +8018,7 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>FIL-GET-03</t>
+          <t>FIL-GET-02</t>
         </is>
       </c>
       <c r="B125" s="12" t="inlineStr">
@@ -8023,19 +8031,19 @@
           <t>GET /api/files/{fileId}</t>
         </is>
       </c>
-      <c r="D125" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D125" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>业务规则</t>
+          <t>异常</t>
         </is>
       </c>
       <c r="F125" s="5" t="inlineStr">
         <is>
-          <t>文件已逻辑删除</t>
+          <t>fileId 不存在</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -8045,7 +8053,7 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>/api/files/{fileId}</t>
+          <t>/api/files/not-exist</t>
         </is>
       </c>
       <c r="I125" s="5" t="inlineStr"/>
@@ -8057,7 +8065,7 @@
       </c>
       <c r="L125" s="5" t="inlineStr">
         <is>
-          <t>DELETED 记录不可查询</t>
+          <t>“文件不存在”</t>
         </is>
       </c>
       <c r="M125" s="5" t="inlineStr"/>
@@ -8065,7 +8073,7 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>FIL-DL-01</t>
+          <t>FIL-GET-03</t>
         </is>
       </c>
       <c r="B126" s="12" t="inlineStr">
@@ -8075,22 +8083,22 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>GET /api/files/{fileId}/download</t>
-        </is>
-      </c>
-      <c r="D126" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>GET /api/files/{fileId}</t>
+        </is>
+      </c>
+      <c r="D126" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>业务规则</t>
         </is>
       </c>
       <c r="F126" s="5" t="inlineStr">
         <is>
-          <t>存在 NORMAL 文件</t>
+          <t>文件已逻辑删除</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -8100,19 +8108,19 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>/api/files/{fileId}/download</t>
+          <t>/api/files/{fileId}</t>
         </is>
       </c>
       <c r="I126" s="5" t="inlineStr"/>
       <c r="J126" s="5" t="inlineStr"/>
       <c r="K126" s="2" t="inlineStr">
         <is>
-          <t>302</t>
+          <t>404</t>
         </is>
       </c>
       <c r="L126" s="5" t="inlineStr">
         <is>
-          <t>返回 302 + Location（MinIO 签名下载地址）</t>
+          <t>DELETED 记录不可查询</t>
         </is>
       </c>
       <c r="M126" s="5" t="inlineStr"/>
@@ -8120,7 +8128,7 @@
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>FIL-DL-02</t>
+          <t>FIL-DL-01</t>
         </is>
       </c>
       <c r="B127" s="12" t="inlineStr">
@@ -8133,19 +8141,19 @@
           <t>GET /api/files/{fileId}/download</t>
         </is>
       </c>
-      <c r="D127" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>异常</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F127" s="5" t="inlineStr">
         <is>
-          <t>fileId 不存在</t>
+          <t>存在 NORMAL 文件</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -8155,19 +8163,19 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>/api/files/not-exist/download</t>
+          <t>/api/files/{fileId}/download</t>
         </is>
       </c>
       <c r="I127" s="5" t="inlineStr"/>
       <c r="J127" s="5" t="inlineStr"/>
       <c r="K127" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>302</t>
         </is>
       </c>
       <c r="L127" s="5" t="inlineStr">
         <is>
-          <t>“文件不存在”</t>
+          <t>返回 302 + Location（MinIO 签名下载地址）</t>
         </is>
       </c>
       <c r="M127" s="5" t="inlineStr"/>
@@ -8175,7 +8183,7 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>FIL-DL-03</t>
+          <t>FIL-DL-02</t>
         </is>
       </c>
       <c r="B128" s="12" t="inlineStr">
@@ -8188,19 +8196,19 @@
           <t>GET /api/files/{fileId}/download</t>
         </is>
       </c>
-      <c r="D128" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D128" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>业务规则</t>
+          <t>异常</t>
         </is>
       </c>
       <c r="F128" s="5" t="inlineStr">
         <is>
-          <t>文件已删除</t>
+          <t>fileId 不存在</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -8210,7 +8218,7 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>/api/files/{fileId}/download</t>
+          <t>/api/files/not-exist/download</t>
         </is>
       </c>
       <c r="I128" s="5" t="inlineStr"/>
@@ -8222,7 +8230,7 @@
       </c>
       <c r="L128" s="5" t="inlineStr">
         <is>
-          <t>DELETED 不可下载</t>
+          <t>“文件不存在”</t>
         </is>
       </c>
       <c r="M128" s="5" t="inlineStr"/>
@@ -8230,7 +8238,7 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>FIL-FDEL-01</t>
+          <t>FIL-DL-03</t>
         </is>
       </c>
       <c r="B129" s="12" t="inlineStr">
@@ -8240,56 +8248,52 @@
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>POST /api/files/{fileId}/delete</t>
-        </is>
-      </c>
-      <c r="D129" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>GET /api/files/{fileId}/download</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>业务规则</t>
         </is>
       </c>
       <c r="F129" s="5" t="inlineStr">
         <is>
-          <t>存在 NORMAL 文件</t>
+          <t>文件已删除</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>/api/files/{fileId}/delete</t>
+          <t>/api/files/{fileId}/download</t>
         </is>
       </c>
       <c r="I129" s="5" t="inlineStr"/>
       <c r="J129" s="5" t="inlineStr"/>
       <c r="K129" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="L129" s="5" t="inlineStr">
         <is>
-          <t>deleted=true；记录置 DELETED，提交后清理 MinIO 对象</t>
-        </is>
-      </c>
-      <c r="M129" s="5" t="inlineStr">
-        <is>
-          <t>逻辑删除</t>
-        </is>
-      </c>
+          <t>DELETED 不可下载</t>
+        </is>
+      </c>
+      <c r="M129" s="5" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>FIL-FDEL-02</t>
+          <t>FIL-FDEL-01</t>
         </is>
       </c>
       <c r="B130" s="12" t="inlineStr">
@@ -8302,19 +8306,19 @@
           <t>POST /api/files/{fileId}/delete</t>
         </is>
       </c>
-      <c r="D130" s="6" t="inlineStr">
-        <is>
-          <t>P1</t>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>异常</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F130" s="5" t="inlineStr">
         <is>
-          <t>fileId 不存在</t>
+          <t>存在 NORMAL 文件</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -8324,27 +8328,31 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>/api/files/not-exist/delete</t>
+          <t>/api/files/{fileId}/delete</t>
         </is>
       </c>
       <c r="I130" s="5" t="inlineStr"/>
       <c r="J130" s="5" t="inlineStr"/>
       <c r="K130" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L130" s="5" t="inlineStr">
         <is>
-          <t>“文件不存在”</t>
-        </is>
-      </c>
-      <c r="M130" s="5" t="inlineStr"/>
+          <t>deleted=true；记录置 DELETED，提交后清理 MinIO 对象</t>
+        </is>
+      </c>
+      <c r="M130" s="5" t="inlineStr">
+        <is>
+          <t>逻辑删除</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>FIL-FDEL-03</t>
+          <t>FIL-FDEL-02</t>
         </is>
       </c>
       <c r="B131" s="12" t="inlineStr">
@@ -8357,19 +8365,19 @@
           <t>POST /api/files/{fileId}/delete</t>
         </is>
       </c>
-      <c r="D131" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>业务规则</t>
+          <t>异常</t>
         </is>
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
-          <t>重复删除同一文件</t>
+          <t>fileId 不存在</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -8379,7 +8387,7 @@
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>/api/files/{fileId}/delete</t>
+          <t>/api/files/not-exist/delete</t>
         </is>
       </c>
       <c r="I131" s="5" t="inlineStr"/>
@@ -8391,7 +8399,7 @@
       </c>
       <c r="L131" s="5" t="inlineStr">
         <is>
-          <t>已 DELETED 不再命中 NORMAL → 404</t>
+          <t>“文件不存在”</t>
         </is>
       </c>
       <c r="M131" s="5" t="inlineStr"/>
@@ -8399,7 +8407,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>FIL-FP-01</t>
+          <t>FIL-FDEL-03</t>
         </is>
       </c>
       <c r="B132" s="12" t="inlineStr">
@@ -8409,22 +8417,22 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>POST /api/files/page</t>
-        </is>
-      </c>
-      <c r="D132" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>POST /api/files/{fileId}/delete</t>
+        </is>
+      </c>
+      <c r="D132" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>正常</t>
+          <t>业务规则</t>
         </is>
       </c>
       <c r="F132" s="5" t="inlineStr">
         <is>
-          <t>存在 NORMAL 文件</t>
+          <t>重复删除同一文件</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -8434,23 +8442,19 @@
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>/api/files/page</t>
+          <t>/api/files/{fileId}/delete</t>
         </is>
       </c>
       <c r="I132" s="5" t="inlineStr"/>
-      <c r="J132" s="5" t="inlineStr">
-        <is>
-          <t>{"pageNo":1,"pageSize":10}</t>
-        </is>
-      </c>
+      <c r="J132" s="5" t="inlineStr"/>
       <c r="K132" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="L132" s="5" t="inlineStr">
         <is>
-          <t>返回 total/pageNo/pageSize/records（仅 NORMAL）</t>
+          <t>已 DELETED 不再命中 NORMAL → 404</t>
         </is>
       </c>
       <c r="M132" s="5" t="inlineStr"/>
@@ -8458,7 +8462,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>FIL-FP-02</t>
+          <t>FIL-FP-01</t>
         </is>
       </c>
       <c r="B133" s="12" t="inlineStr">
@@ -8471,9 +8475,9 @@
           <t>POST /api/files/page</t>
         </is>
       </c>
-      <c r="D133" s="8" t="inlineStr">
-        <is>
-          <t>P2</t>
+      <c r="D133" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
@@ -8483,7 +8487,7 @@
       </c>
       <c r="F133" s="5" t="inlineStr">
         <is>
-          <t>按名称/扩展名过滤</t>
+          <t>存在 NORMAL 文件</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -8499,7 +8503,7 @@
       <c r="I133" s="5" t="inlineStr"/>
       <c r="J133" s="5" t="inlineStr">
         <is>
-          <t>{"originalName":"demo","fileExt":"zip"}</t>
+          <t>{"pageNo":1,"pageSize":10}</t>
         </is>
       </c>
       <c r="K133" s="2" t="inlineStr">
@@ -8509,7 +8513,7 @@
       </c>
       <c r="L133" s="5" t="inlineStr">
         <is>
-          <t>按 originalName/fileExt 可选过滤</t>
+          <t>返回 total/pageNo/pageSize/records（仅 NORMAL）</t>
         </is>
       </c>
       <c r="M133" s="5" t="inlineStr"/>
@@ -8517,7 +8521,7 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>FIL-FP-03</t>
+          <t>FIL-FP-02</t>
         </is>
       </c>
       <c r="B134" s="12" t="inlineStr">
@@ -8537,12 +8541,12 @@
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>边界</t>
+          <t>正常</t>
         </is>
       </c>
       <c r="F134" s="5" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>按名称/扩展名过滤</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -8558,7 +8562,7 @@
       <c r="I134" s="5" t="inlineStr"/>
       <c r="J134" s="5" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t>{"originalName":"demo","fileExt":"zip"}</t>
         </is>
       </c>
       <c r="K134" s="2" t="inlineStr">
@@ -8568,19 +8572,15 @@
       </c>
       <c r="L134" s="5" t="inlineStr">
         <is>
-          <t>pageNo=1，pageSize 缺省=20</t>
-        </is>
-      </c>
-      <c r="M134" s="5" t="inlineStr">
-        <is>
-          <t>缺省分页</t>
-        </is>
-      </c>
+          <t>按 originalName/fileExt 可选过滤</t>
+        </is>
+      </c>
+      <c r="M134" s="5" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>FIL-FP-04</t>
+          <t>FIL-FP-03</t>
         </is>
       </c>
       <c r="B135" s="12" t="inlineStr">
@@ -8621,23 +8621,86 @@
       <c r="I135" s="5" t="inlineStr"/>
       <c r="J135" s="5" t="inlineStr">
         <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="L135" s="5" t="inlineStr">
+        <is>
+          <t>pageNo=1，pageSize 缺省=20</t>
+        </is>
+      </c>
+      <c r="M135" s="5" t="inlineStr">
+        <is>
+          <t>缺省分页</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>FIL-FP-04</t>
+        </is>
+      </c>
+      <c r="B136" s="12" t="inlineStr">
+        <is>
+          <t>文件上传中心</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/files/page</t>
+        </is>
+      </c>
+      <c r="D136" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>边界</t>
+        </is>
+      </c>
+      <c r="F136" s="5" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>/api/files/page</t>
+        </is>
+      </c>
+      <c r="I136" s="5" t="inlineStr"/>
+      <c r="J136" s="5" t="inlineStr">
+        <is>
           <t>{"pageNo":0,"pageSize":9999}</t>
         </is>
       </c>
-      <c r="K135" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="L135" s="5" t="inlineStr">
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="L136" s="5" t="inlineStr">
         <is>
           <t>pageNo=1；pageSize 受 max-page-size(100) 限制</t>
         </is>
       </c>
-      <c r="M135" s="5" t="inlineStr"/>
+      <c r="M136" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M135"/>
+  <autoFilter ref="A1:M136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10449,7 +10512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10526,7 +10589,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_UNAUTHORIZED","message":"请先登录","data":null,"traceId":"4bbd46e70e7b4d8882cfdcef5855111b","timestamp":"2026-08-17T11:33:44.364"}</t>
+          <t>{"success":false,"code":"COMMON_UNAUTHORIZED","message":"请先登录","data":null,"traceId":"41952a64d7b3444e958670452e70efa7","timestamp":"2026-08-18T09:50:45.674"}</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -10563,7 +10626,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"count":1200006},"traceId":"ee5bc1ba8f764019bfbfa09a2878e561","timestamp":"2026-08-17T11:33:44.883"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"count":2300019},"traceId":"14e4f46d0ed240969741d9bb8fdb1e9e","timestamp":"2026-08-18T09:50:46.254"}</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
@@ -10596,7 +10659,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":3,"count":1200009,"elapsedMs":185},"traceId":"79e06370ab004ddbab3e0ffd9fdcc1b3","timestamp":"2026-08-17T11:33:45.527"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":3,"count":2300022,"elapsedMs":378},"traceId":"10f1789d5e3841adac77a9c3ceb6c8b7","timestamp":"2026-08-18T09:50:47.212"}</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr"/>
@@ -10629,7 +10692,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":0,"count":1200009,"elapsedMs":170},"traceId":"5240daeea9ad404ba6aedeb3a5b8092d","timestamp":"2026-08-17T11:33:46.236"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":0,"count":2300022,"elapsedMs":342},"traceId":"b0511b608ebf4ff8a12ece1472bcf075","timestamp":"2026-08-18T09:50:48.071"}</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr"/>
@@ -10652,17 +10715,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>❌ FAIL</t>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>✅ PASS</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_INTERNAL_ERROR","message":"服务内部异常","data":null,"traceId":"5fc1da9e4b3c44d7b00ab9209c134f44","timestamp":"2026-08-17T11:33:46.46"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求参数类型错误","data":null,"traceId":"29ed933ff0614380b4c9850514d9ea99","timestamp":"2026-08-18T09:50:48.304"}</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
@@ -10695,7 +10758,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>PK7\][Content_Types].xml�S�n�0����*6�PU�C���\{�X�%����]8�R� q�cfgfW�d�q�ZCB|��|�*�*h㻆},^�{Va�^K&lt;4�6�N�XQ�ǆ�9�!P��$��҆�d�c�D�j);��ѝP�g��E�M'O�ʕ����H7L�h���R���G��^�'�{��zސʮB��3�˙��h.�h�W�жF�j娄C …</t>
+          <t>PKXN][Content_Types].xml�S�n�0����*6�PU�C���\{�X�%����]8�R� q�cfgfW�d�q�ZCB|��|�*�*h㻆},^�{Va�^K&lt;4�6�N�XQ�ǆ�9�!P��$��҆�d�c�D�j);��ѝP�g��E�M'O�ʕ����H7L�h���R���G��^�'�{��zސʮB��3�˙��h.�h�W�жF�j娄C …</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -10732,7 +10795,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"c42eac2147554ec792c6784c4db0c678","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"bb710d51fd834e2b880bbf6c0eefa695","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr"/>
@@ -10765,7 +10828,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"c42eac2147554ec792c6784c4db0c678","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"totalCount":3,"completedCount":3,"retryCount":0,"maxRetryCount":3,"errorMe …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"bb710d51fd834e2b880bbf6c0eefa695","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"totalCount":3,"completedCount":3,"retryCount":0,"maxRetryCount":3,"errorMe …</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -10802,7 +10865,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入任务不存在","data":null,"traceId":"352d6a875622487985c70c66cef6b5ef","timestamp":"2026-08-17T11:33:50.529"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入任务不存在","data":null,"traceId":"1ef67b909f2a4c2c8790466c3d87573b","timestamp":"2026-08-18T09:50:53.453"}</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr"/>
@@ -10835,7 +10898,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入错误明细文件不存在","data":null,"traceId":"40e6387503c34c9fa66c818094921acd","timestamp":"2026-08-17T11:33:50.746"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入错误明细文件不存在","data":null,"traceId":"ae7960ed59f34d2396d288647d9fc876","timestamp":"2026-08-18T09:50:53.661"}</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
@@ -10858,17 +10921,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>❌ FAIL</t>
+          <t>415</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>✅ PASS</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_INTERNAL_ERROR","message":"服务内部异常","data":null,"traceId":"41d8ca4baf9b4c94abc37705c0f66c3a","timestamp":"2026-08-17T11:33:50.955"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"cf6679483a7a4fe6bb326860e7b652d8","timestamp":"2026-08-18T09:50:53.856"}</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr"/>
@@ -10901,7 +10964,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件不能为空","data":null,"traceId":"afedf6c392a54ecb8e8948d8513b6f20","timestamp":"2026-08-17T11:33:51.153"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件不能为空","data":null,"traceId":"ae79dfad00a04163a8ba436dbb665362","timestamp":"2026-08-18T09:50:54.038"}</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr"/>
@@ -10919,12 +10982,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -10934,12 +10997,12 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"06bb5a71981f47bf9d1c9a81f67e817d","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件格式错误，请上传 .xlsx 文件","data":null,"traceId":"0c758b49993d46a58534a19179881537","timestamp":"2026-08-18T09:50:54.277"}</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>提交返回 taskId，异步解析应 FAILED</t>
+          <t>提交阶段校验文件头和 xlsx 结构，非法文件不创建异步任务</t>
         </is>
       </c>
     </row>
@@ -10971,7 +11034,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"09feb86b887f4ba0910cd765d28d5686","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr"/>
@@ -11004,7 +11067,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"e70b17a7aee04e6fb0542f3b8da8a7c0","canceled":true},"traceId":"4aea29c0beac4c0196e6c3869852c7c8","timestamp":"2026-08-17T11:33:54.242"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"a77b0f4392714386bf94ed7e17908f61","canceled":true},"traceId":"84113fe782624895bf6616f87a965426","timestamp":"2026-08-18T09:50:55.027"}</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -11037,7 +11100,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"09feb86b887f4ba0910cd765d28d5686","ownerId":"user-1","status":"FAILED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","status":"FAILED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -11074,7 +11137,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>{"timestamp":"2026-08-17T03:33:54.643+00:00","status":404,"error":"Not Found","path":"/api/excel/not-exist"}</t>
+          <t>{"timestamp":"2026-08-18T01:50:57.647+00:00","status":404,"error":"Not Found","path":"/api/excel/not-exist"}</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
@@ -11107,7 +11170,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"78bf2a95a1f84636af82c6b0369b7490","timestamp":"2026-08-17T11:33:54.835"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"dc3944f6a2a34889b8dd06b2fcc9c6a7","timestamp":"2026-08-18T09:50:57.894"}</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr"/>
@@ -11125,7 +11188,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>302</t>
+          <t>409</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -11133,19 +11196,19 @@
           <t>409</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>❌ FAIL</t>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>✅ PASS</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"导出任务尚未完成","data":null,"traceId":"90ec7a3b632c40e4a278f3c90638e05b","timestamp":"2026-08-17T11:33:55.106"}</t>
+          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"导出任务尚未完成","data":null,"traceId":"5098f04395ea4776a8732ff42fb2443c","timestamp":"2026-08-18T09:50:58.096"}</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>正确边界：1,200,009 行 &gt; 单 Sheet 上限 1,048,575，导出任务按设计失败（E-03 实测验证）</t>
+          <t>导出任务状态=FAILED；SUCCESS 才应 302，FAILED/CANCELED/未完成应 409</t>
         </is>
       </c>
     </row>
@@ -11177,7 +11240,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"ad730f358f2646b2bfba0ccc3c788f4c","timestamp":"2026-08-17T11:33:55.326"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"f643b97d4bf141eab6c2bfac8e43612e","timestamp":"2026-08-18T09:50:58.284"}</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
@@ -11210,7 +11273,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":14,"pageNo":1,"pageSize":5,"records":[{"taskId":"09feb86b887f4ba0910cd765d28d5686","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"a7b5e375b86e49 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":32,"pageNo":1,"pageSize":5,"records":[{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"59dcbfe6a79a4d …</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
@@ -11243,7 +11306,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":14,"pageNo":1,"pageSize":20,"records":[{"taskId":"09feb86b887f4ba0910cd765d28d5686","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"a7b5e375b86e4 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":32,"pageNo":1,"pageSize":20,"records":[{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"59dcbfe6a79a4 …</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr"/>
@@ -11276,7 +11339,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":14,"pageNo":1,"pageSize":100,"records":[{"taskId":"09feb86b887f4ba0910cd765d28d5686","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"a7b5e375b86e …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":32,"pageNo":1,"pageSize":100,"records":[{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"59dcbfe6a79a …</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr"/>
@@ -11309,7 +11372,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskStatus.GARBAGE","data":null,"traceId":"22317fc475d044cc8c4600cbd8ef2ff3","timestamp":"2026-08-17T11:33:56.211"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskStatus.GARBAGE","data":null,"traceId":"88bca51dd90d4e9393ec8e0e71875ea0","timestamp":"2026-08-18T09:50:59.663"}</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -11346,7 +11409,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskType.GARBAGE","data":null,"traceId":"8ee693a50b1b408b8d8d7cd15298d401","timestamp":"2026-08-17T11:33:56.427"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskType.GARBAGE","data":null,"traceId":"f1ffe2deae2e42038a516c36cc8813aa","timestamp":"2026-08-18T09:50:59.842"}</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -11383,7 +11446,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"09feb86b887f4ba0910cd765d28d5686","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"a7b5e375b86e49928039afe8d22292aa","status":"FAILED","progress …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"59dcbfe6a79a4d758901c2dd62f53623","status":"FAILED","progress …</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr"/>
@@ -11416,7 +11479,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"0f2ac3aeb6644609bc3bdbb80dbe620e","timestamp":"2026-08-17T11:33:56.831"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"4401ae82539c4a6eb6a261ebb955187b","timestamp":"2026-08-18T09:51:00.227"}</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
@@ -11449,7 +11512,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"f1085a30cd214b72a21d8d5bfddb064c","timestamp":"2026-08-17T11:33:57.028"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"0df794a4ebd048dba72fc646e1e307ed","timestamp":"2026-08-18T09:51:00.428"}</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
@@ -11482,7 +11545,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"09feb86b887f4ba0910cd765d28d5686","canceled":false},"traceId":"5b7b305f780d41fabbfc9de8ece6269c","timestamp":"2026-08-17T11:33:57.243"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","canceled":false},"traceId":"058c2964ac5b45d7b8cda02956663050","timestamp":"2026-08-18T09:51:00.687"}</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -11499,12 +11562,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>/api/tasks/{taskId}/retry (SUCCESS)</t>
+          <t>/api/tasks/{taskId}/retry (terminal)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -11512,19 +11575,19 @@
           <t>200</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>❌ FAIL</t>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>✅ PASS</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"09feb86b887f4ba0910cd765d28d5686","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"a7b5e375b86e49928039afe8d22292aa","status":"CREATED","progres …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"59dcbfe6a79a4d758901c2dd62f53623","status":"CREATED","progres …</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>正确行为：该任务为 FAILED 可重试，返回 200</t>
+          <t>重试前任务状态=FAILED；FAILED/CANCELED/EXPIRED 应 200，其余应 409</t>
         </is>
       </c>
     </row>
@@ -11556,7 +11619,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"f6e64831d8f34f9394c725be56fc8474","timestamp":"2026-08-17T11:33:57.684"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"2a6d3fc5caec4aa181432be5e4d9ed93","timestamp":"2026-08-18T09:51:01.184"}</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr"/>
@@ -11589,10 +11652,14 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"e70b17a7aee04e6fb0542f3b8da8a7c0","ownerId":"admin","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"d5abb342b776409892d01bf04ead2598","status":"CREATED","progress …</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr"/>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"a77b0f4392714386bf94ed7e17908f61","ownerId":"admin","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"0c86e89a083f4beba6c6ef4dc66ddcd6","status":"CREATED","progress …</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>重试前任务状态=CANCELED；空库或小数据量下取消可能来晚，若已 SUCCESS 则 409 为正确行为</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -11622,7 +11689,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"b9e51b7a8a884da2a91dfa6c0b2f8e6b","ownerId":"user-1","runControlCode":"RT86937637","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"c8baaec8b27b4ab59d32531dc7a8ec41","ownerId":"user-1","runControlCode":"RT87017861","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr"/>
@@ -11655,7 +11722,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码不能为空","data":null,"traceId":"c5a7e3f7414b45ca9c84a8f75c90d3e7","timestamp":"2026-08-17T11:33:58.435"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码不能为空","data":null,"traceId":"3d31e5dbde4a445db581798d3d9ce797","timestamp":"2026-08-18T09:51:02.125"}</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr"/>
@@ -11688,7 +11755,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码已存在","data":null,"traceId":"bba185a107c547588dd46300b2a2c97e","timestamp":"2026-08-17T11:33:58.69"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码已存在","data":null,"traceId":"138c828be7004621bf0249240fdd6893","timestamp":"2026-08-18T09:51:02.319"}</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr"/>
@@ -11721,7 +11788,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄必须在0到150之间","data":null,"traceId":"8d1fb7a4667242619f223d6aae9622f7","timestamp":"2026-08-17T11:33:58.871"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄必须在0到150之间","data":null,"traceId":"6c3965f2605f4656b1e4eb115dbb31b8","timestamp":"2026-08-18T09:51:02.528"}</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr"/>
@@ -11754,7 +11821,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最大年龄必须在0到150之间","data":null,"traceId":"b74325d6a62d452f90c3926d377b10d8","timestamp":"2026-08-17T11:33:59.094"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最大年龄必须在0到150之间","data":null,"traceId":"fa793155b2a34db5b4131747b0ffddf6","timestamp":"2026-08-18T09:51:02.761"}</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
@@ -11787,7 +11854,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"367cde88874f47409e95960ccdd7dfdc","timestamp":"2026-08-17T11:33:59.31"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"836c24f810fd4bcb9e260dc020fc7dcb","timestamp":"2026-08-18T09:51:03.016"}</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr"/>
@@ -11820,7 +11887,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"runId":"b9e51b7a8a884da2a91dfa6c0b2f8e6b","ownerId":"user-1","runControlCode":"RT86937637","runName":"2026春季测试","studentNo":"T202608 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"runId":"c8baaec8b27b4ab59d32531dc7a8ec41","ownerId":"user-1","runControlCode":"RT87017861","runName":"2026春季测试","studentNo":"T202608 …</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr"/>
@@ -11853,7 +11920,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.excel.domain.model.StudentReportRunStatus.GARBAGE","data":null,"traceId":"7c64d67631884f45a35866159fcb08b6","timestamp":"2026-08-17T11:33:59.702"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.excel.domain.model.StudentReportRunStatus.GARBAGE","data":null,"traceId":"ae1dbacd908b449bb19ce1f04bb895b9","timestamp":"2026-08-18T09:51:03.462"}</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -11890,7 +11957,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"b9e51b7a8a884da2a91dfa6c0b2f8e6b","ownerId":"user-1","runControlCode":"RT86937637","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"c8baaec8b27b4ab59d32531dc7a8ec41","ownerId":"user-1","runControlCode":"RT87017861","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
@@ -11923,7 +11990,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"40d6caef3c7e4c3187c35b886d3f4e98","timestamp":"2026-08-17T11:34:00.056"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"804ef8dbb176422d9c658036963f7767","timestamp":"2026-08-18T09:51:03.909"}</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr"/>
@@ -11956,7 +12023,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"81c2022570bd44acbf372dc84dbc2c1a","timestamp":"2026-08-17T11:34:00.267"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"f8a86b57aed745b280ce44858f556d61","timestamp":"2026-08-18T09:51:04.1"}</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr"/>
@@ -11989,7 +12056,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"b9e51b7a8a884da2a91dfa6c0b2f8e6b","ownerId":"user-1","runControlCode":"RT86937637","runName":"2026春季改","studentNo":null,"nameKeyword":null,"className":"一班","gender":null, …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"c8baaec8b27b4ab59d32531dc7a8ec41","ownerId":"user-1","runControlCode":"RT87017861","runName":"2026春季改","studentNo":null,"nameKeyword":null,"className":"一班","gender":null, …</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr"/>
@@ -12022,7 +12089,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"4adfd9a89dc04a98908656d4e367fe98","timestamp":"2026-08-17T11:34:00.692"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"fe8382a2f7574814a1599fd20c537b26","timestamp":"2026-08-18T09:51:04.49"}</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr"/>
@@ -12055,7 +12122,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"68ce2a378bfd4094b3830114a70aa8b6","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"7c058027f41a4b7984ed0856d1c5b065","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr"/>
@@ -12088,7 +12155,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"taskId":"68ce2a378bfd4094b3830114a70aa8b6","ownerId":"user-1","taskType":"EXPORT","taskName":"学生报表导出-2026春季改","businessKey":"b9e51b7 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"taskId":"7c058027f41a4b7984ed0856d1c5b065","ownerId":"user-1","taskType":"EXPORT","taskName":"学生报表导出-2026春季改","businessKey":"c8baaec …</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr"/>
@@ -12121,7 +12188,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"b9e51b7a8a884da2a91dfa6c0b2f8e6b","deleted":true},"traceId":"5e79a89d2d2741128da36dcf44771c12","timestamp":"2026-08-17T11:34:01.852"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"c8baaec8b27b4ab59d32531dc7a8ec41","deleted":true},"traceId":"0ba044c2ad474632a9028b594e6f45cb","timestamp":"2026-08-18T09:51:05.978"}</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr"/>
@@ -12154,7 +12221,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"90f6f49b50544323ada3706da6a62d38","timestamp":"2026-08-17T11:34:02.067"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"57f4cb73a7964ca4898e256b6cc26cf6","timestamp":"2026-08-18T09:51:06.163"}</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr"/>
@@ -12187,7 +12254,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"04ee98430ab2474c90e92b6a9339d3d4","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fileExt":"txt","statu …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"1bbf7dd099874d3698f4f6ada1e595f2","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fileExt":"txt","statu …</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr"/>
@@ -12210,17 +12277,17 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>❌ FAIL</t>
+          <t>415</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>✅ PASS</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_INTERNAL_ERROR","message":"服务内部异常","data":null,"traceId":"9f4b6f5d726f4e99b5b02511c89018c6","timestamp":"2026-08-17T11:34:02.676"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"36f427f4ce53474f97e0badcc3caf959","timestamp":"2026-08-18T09:51:06.547"}</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr"/>
@@ -12253,7 +12320,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"上传文件不能为空","data":null,"traceId":"2b7d2144ff0842bb936daedf4bfe1760","timestamp":"2026-08-17T11:34:02.958"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"上传文件不能为空","data":null,"traceId":"9e35522f393848a6bc32ed7adeb724b2","timestamp":"2026-08-18T09:51:06.739"}</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr"/>
@@ -12261,22 +12328,22 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>FIL-IC-01</t>
+          <t>FIL-UP-04</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>/api/files/instant-check (hit)</t>
+          <t>/api/files/upload (fake executable xlsx)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -12286,20 +12353,24 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":true,"file":{"fileId":"04ee98430ab2474c90e92b6a9339d3d4","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d …</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr"/>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件内容疑似可执行程序，originalName=evil.xlsx","data":null,"traceId":"4408cfb28ea84198af6b63788c32afc4","timestamp":"2026-08-18T09:51:06.957"}</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>文件安全扫描：内容嗅探拦截伪装可执行文件 ✅</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>FIL-IC-02</t>
+          <t>FIL-IC-01</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>/api/files/instant-check (miss)</t>
+          <t>/api/files/instant-check (hit)</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -12319,7 +12390,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":false,"file":null},"traceId":"ed261e67165349e495d0f4b4fa0bdad8","timestamp":"2026-08-17T11:34:03.466"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":true,"file":{"fileId":"1bbf7dd099874d3698f4f6ada1e595f2","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d …</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr"/>
@@ -12327,22 +12398,22 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>FIL-IC-03</t>
+          <t>FIL-IC-02</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>/api/files/instant-check (no md5)</t>
+          <t>/api/files/instant-check (miss)</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -12352,7 +12423,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 不能为空","data":null,"traceId":"595919ecaa25498f97d48bc1564e360f","timestamp":"2026-08-17T11:34:03.69"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":false,"file":null},"traceId":"1ad5344e60644569a8304d74f55b87a5","timestamp":"2026-08-18T09:51:07.491"}</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr"/>
@@ -12360,12 +12431,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>FIL-IC-04</t>
+          <t>FIL-IC-03</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>/api/files/instant-check (bad md5)</t>
+          <t>/api/files/instant-check (no md5)</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -12385,7 +12456,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"e8debb0605714d9fb62a7a886cfc51b8","timestamp":"2026-08-17T11:34:03.956"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 不能为空","data":null,"traceId":"6a46098c28b94cfba78660dc5b40862f","timestamp":"2026-08-18T09:51:07.727"}</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr"/>
@@ -12393,12 +12464,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>FIL-IC-05</t>
+          <t>FIL-IC-04</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>/api/files/instant-check (size 0)</t>
+          <t>/api/files/instant-check (bad md5)</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -12418,7 +12489,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件大小必须大于 0","data":null,"traceId":"8a8cabb7b82f43dfb82021809d08465e","timestamp":"2026-08-17T11:34:04.15"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"55e12b30dcbb462ba44719c36a043bdf","timestamp":"2026-08-18T09:51:07.947"}</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr"/>
@@ -12426,22 +12497,22 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>FIL-GET-01</t>
+          <t>FIL-IC-05</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>/api/files/{fileId}</t>
+          <t>/api/files/instant-check (size 0)</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -12451,7 +12522,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"04ee98430ab2474c90e92b6a9339d3d4","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fi …</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件大小必须大于 0","data":null,"traceId":"c7a177741ba8495da784002f496c9cdc","timestamp":"2026-08-18T09:51:08.233"}</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr"/>
@@ -12459,22 +12530,22 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>FIL-GET-02</t>
+          <t>FIL-GET-01</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>/api/files/not-exist</t>
+          <t>/api/files/{fileId}</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
@@ -12484,7 +12555,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"d8ea69930cc248fb9db9de331739349e","timestamp":"2026-08-17T11:34:04.552"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"1bbf7dd099874d3698f4f6ada1e595f2","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fi …</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr"/>
@@ -12492,22 +12563,22 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>FIL-FP-01</t>
+          <t>FIL-GET-02</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>/api/files/page</t>
+          <t>/api/files/not-exist</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -12517,7 +12588,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":2,"pageNo":1,"pageSize":5,"records":[{"fileId":"04ee98430ab2474c90e92b6a9339d3d4","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"f …</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"557d7598ef5b49df967243322a8f45f9","timestamp":"2026-08-18T09:51:08.653"}</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr"/>
@@ -12525,22 +12596,22 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>FIL-DL-01</t>
+          <t>FIL-FP-01</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>/api/files/{fileId}/download</t>
+          <t>/api/files/page</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>302</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>302</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
@@ -12548,28 +12619,32 @@
           <t>✅ PASS</t>
         </is>
       </c>
-      <c r="F62" s="5" t="inlineStr"/>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":8,"pageNo":1,"pageSize":5,"records":[{"fileId":"1bbf7dd099874d3698f4f6ada1e595f2","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"f …</t>
+        </is>
+      </c>
       <c r="G62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>FIL-DL-02</t>
+          <t>FIL-DL-01</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>/api/files/not-exist/download</t>
+          <t>/api/files/{fileId}/download</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>302</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>302</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
@@ -12577,32 +12652,28 @@
           <t>✅ PASS</t>
         </is>
       </c>
-      <c r="F63" s="5" t="inlineStr">
-        <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"36eea08caaba4663ae547a2a643d8f6c","timestamp":"2026-08-17T11:34:05.495"}</t>
-        </is>
-      </c>
+      <c r="F63" s="5" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>FIL-DI-01</t>
+          <t>FIL-DL-02</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>/api/files/direct/init</t>
+          <t>/api/files/not-exist/download</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -12612,7 +12683,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":true,"uploadId":null,"fileId":"04ee98430ab2474c90e92b6a9339d3d4","uploadUrl":null,"objectKey":null,"expireMinutes":null,"file":{"fileId":"04ee98430ab2474c90e92b6a9339d3d …</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"ce1509874776456a94cc064cef119a15","timestamp":"2026-08-18T09:51:09.637"}</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr"/>
@@ -12620,22 +12691,22 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>FIL-DI-04</t>
+          <t>FIL-DI-01</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>/api/files/direct/init (bad md5)</t>
+          <t>/api/files/direct/init</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -12645,7 +12716,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"a7ea6cc186e5499ca1485ee3e31124e0","timestamp":"2026-08-17T11:34:06.029"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":true,"uploadId":null,"fileId":"1bbf7dd099874d3698f4f6ada1e595f2","uploadUrl":null,"objectKey":null,"expireMinutes":null,"file":{"fileId":"1bbf7dd099874d3698f4f6ada1e595f …</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr"/>
@@ -12653,22 +12724,22 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>FIL-DC-02</t>
+          <t>FIL-DI-04</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>/api/files/direct/not-exist/complete</t>
+          <t>/api/files/direct/init (bad md5)</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>400</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>400</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
@@ -12678,7 +12749,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"822a2e39717340b68c4df5f4e61d0a44","timestamp":"2026-08-17T11:34:06.293"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"2ba416c64658459a8600e8a0fab4ddbd","timestamp":"2026-08-18T09:51:10.132"}</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr"/>
@@ -12686,22 +12757,22 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>FIL-MI-01</t>
+          <t>FIL-DC-02</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>/api/files/multipart/init</t>
+          <t>/api/files/direct/not-exist/complete</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -12711,7 +12782,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"560d8cdfa64a4b9a910d268c1c66bf4b","fileId":"d735d530f76040e798beaef1e2e98621","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"050c1f700349417fb8fd277cebc6101c","timestamp":"2026-08-18T09:51:10.416"}</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr"/>
@@ -12719,12 +12790,12 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>FIL-MP-01</t>
+          <t>FIL-MI-01</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>/api/files/multipart/{uploadId}/parts</t>
+          <t>/api/files/multipart/init</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -12744,24 +12815,20 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"uploadId":"560d8cdfa64a4b9a910d268c1c66bf4b","partCount":3,"uploadedParts":[1,2]},"traceId":"c7c50e8df10540be820051aa982b12c7","timestamp":"2026-08-17T11:35:42.595"}</t>
-        </is>
-      </c>
-      <c r="G68" s="5" t="inlineStr">
-        <is>
-          <t>期望 uploadedParts 含已传分片</t>
-        </is>
-      </c>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"7830734486bf4a25bb95170d6438b887","fileId":"a834328e39ac41b6b10660af4c826bea","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>FIL-MC-01</t>
+          <t>FIL-MP-01</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>/api/files/multipart/{uploadId}/complete</t>
+          <t>/api/files/multipart/{uploadId}/parts</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -12781,30 +12848,34 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"d735d530f76040e798beaef1e2e98621","ownerId":"user-1","originalName":"big.bin","contentType":null,"fileSize":12582912,"fileMd5":"5e39c18e738ce2cb8700c256aac882fd","fileEx …</t>
-        </is>
-      </c>
-      <c r="G69" s="5" t="inlineStr"/>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"uploadId":"7830734486bf4a25bb95170d6438b887","partCount":3,"uploadedParts":[1,2]},"traceId":"940bb22c851441d6be88f4d8c4974c56","timestamp":"2026-08-18T09:52:14.888"}</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>期望 uploadedParts 含已传分片</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>FIL-MP-03</t>
+          <t>FIL-MC-01</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>/api/files/multipart/not-exist/parts</t>
+          <t>/api/files/multipart/{uploadId}/complete</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
@@ -12814,7 +12885,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"4265c3b01c6d4fc796b94060d5665768","timestamp":"2026-08-17T11:36:00.309"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"a834328e39ac41b6b10660af4c826bea","ownerId":"user-1","originalName":"big.bin","contentType":null,"fileSize":12582912,"fileMd5":"825b98cb69356d962a9006a51cbbadff","fileEx …</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr"/>
@@ -12822,22 +12893,22 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>FIL-MA-init</t>
+          <t>FIL-MP-03</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>/api/files/multipart/init (for abort)</t>
+          <t>/api/files/multipart/not-exist/parts</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>404</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
@@ -12847,7 +12918,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"ee451bb878f148db94d65da2ec07f026","fileId":"153f3416c9b1451b8cc0dc4911f8eae5","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"bcb7b2d8c0a74001ba0b182014897d89","timestamp":"2026-08-18T09:52:29.379"}</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr"/>
@@ -12855,12 +12926,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>FIL-MA-01</t>
+          <t>FIL-MA-init</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>/api/files/multipart/{uploadId}/abort</t>
+          <t>/api/files/multipart/init (for abort)</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -12880,7 +12951,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"ee451bb878f148db94d65da2ec07f026"},"traceId":"77fc9e3a0d3044b29fa8fba31206bee7","timestamp":"2026-08-17T11:36:00.969"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"d6dc0c4cc5bb4cfcb82edd8c8d86d930","fileId":"ff0ff84b51a0474584cd5ce193e646f8","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr"/>
@@ -12888,22 +12959,22 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>FIL-MA-02</t>
+          <t>FIL-MA-01</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>/api/files/multipart/{uploadId}/abort (again)</t>
+          <t>/api/files/multipart/{uploadId}/abort</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
@@ -12913,7 +12984,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"上传任务状态不允许完成，status=ABORTED","data":null,"traceId":"b04ba285131d491f82d19f63a4501e67","timestamp":"2026-08-17T11:36:01.262"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"d6dc0c4cc5bb4cfcb82edd8c8d86d930"},"traceId":"abecf29242a74399b62f2800997359fd","timestamp":"2026-08-18T09:52:31.417"}</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr"/>
@@ -12921,22 +12992,22 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>FIL-MI-05</t>
+          <t>FIL-MA-02</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>/api/files/multipart/init (bad md5)</t>
+          <t>/api/files/multipart/{uploadId}/abort (again)</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>409</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>409</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
@@ -12946,7 +13017,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"1b603a763a1040f18aa6f7b390f1412a","timestamp":"2026-08-17T11:36:01.564"}</t>
+          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"上传任务状态不允许完成，status=ABORTED","data":null,"traceId":"ec5651fe434e41daab45623b2dc2b2c9","timestamp":"2026-08-18T09:52:31.891"}</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr"/>
@@ -12954,22 +13025,22 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>FIL-FDEL-01</t>
+          <t>FIL-MI-05</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>/api/files/{fileId}/delete</t>
+          <t>/api/files/multipart/init (bad md5)</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -12979,7 +13050,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"deleted":true,"fileId":"04ee98430ab2474c90e92b6a9339d3d4"},"traceId":"19923d47c469480fac80d79ac98e4924","timestamp":"2026-08-17T11:36:01.816"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"2716cc045d824c0382552132c424e617","timestamp":"2026-08-18T09:52:32.24"}</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr"/>
@@ -12987,22 +13058,22 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>FIL-FDEL-02</t>
+          <t>FIL-FDEL-01</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>/api/files/not-exist/delete</t>
+          <t>/api/files/{fileId}/delete</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
@@ -13012,7 +13083,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"bedf4ef55bd541179b399dd055ffbd2a","timestamp":"2026-08-17T11:36:02.046"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"deleted":true,"fileId":"1bbf7dd099874d3698f4f6ada1e595f2"},"traceId":"d2fa48feab8c4aa88f3debc2e6184aaa","timestamp":"2026-08-18T09:52:32.7"}</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr"/>
@@ -13020,50 +13091,83 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
+          <t>FIL-FDEL-02</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>/api/files/not-exist/delete</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>✅ PASS</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"7ea8fef722e947209bedfd5a739c0676","timestamp":"2026-08-18T09:52:33.033"}</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
           <t>FIL-GET-03</t>
         </is>
       </c>
-      <c r="B77" s="5" t="inlineStr">
+      <c r="B78" s="5" t="inlineStr">
         <is>
           <t>/api/files/{fileId} (deleted)</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>404</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>404</t>
         </is>
       </c>
-      <c r="E77" s="8" t="inlineStr">
+      <c r="E78" s="8" t="inlineStr">
         <is>
           <t>✅ PASS</t>
         </is>
       </c>
-      <c r="F77" s="5" t="inlineStr">
-        <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"f5620ab51c904cbf8b9a0264097d86a5","timestamp":"2026-08-17T11:36:02.229"}</t>
-        </is>
-      </c>
-      <c r="G77" s="5" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="13" t="inlineStr">
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"b355268fe94f4f6f9de3233af816b36a","timestamp":"2026-08-18T09:52:33.582"}</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="13" t="inlineStr">
         <is>
           <t>汇总</t>
         </is>
       </c>
-      <c r="B78" s="13" t="inlineStr">
-        <is>
-          <t>标准环境 R7 加固后复测：总 76  ✅PASS 71  ❌FAIL 5（真实缺陷仅 F-02 三项，2 项为单 Sheet 上限正确边界）</t>
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>标准环境 R11（文件安全扫描版，2026-08-18 09:52）：总 77  ✅PASS 77  ❌FAIL 0 —— 含新增 FIL-UP-04 安全用例</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G77"/>
+  <autoFilter ref="A1:G78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: harden async import export workflows
</commit_message>
<xml_diff>
--- a/docs/test/接口扁平化测试用例.xlsx
+++ b/docs/test/接口扁平化测试用例.xlsx
@@ -9,12 +9,12 @@
   <sheets>
     <sheet name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="接口参数列表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="执行结果(标准环境R11)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="执行结果(标准环境R14)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$M$136</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'接口参数列表'!$A$1:$K$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'执行结果(标准环境R11)'!$A$1:$G$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'执行结果(标准环境R14)'!$A$1:$G$78</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -10589,7 +10589,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_UNAUTHORIZED","message":"请先登录","data":null,"traceId":"41952a64d7b3444e958670452e70efa7","timestamp":"2026-08-18T09:50:45.674"}</t>
+          <t>{"success":false,"code":"COMMON_UNAUTHORIZED","message":"请先登录","data":null,"traceId":"8c7234fa2d59431080dc1548e6e22beb","timestamp":"2026-08-18T20:14:43.744"}</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -10626,7 +10626,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"count":2300019},"traceId":"14e4f46d0ed240969741d9bb8fdb1e9e","timestamp":"2026-08-18T09:50:46.254"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"count":3},"traceId":"ca09c73c5a4245348c98e3c99f84041a","timestamp":"2026-08-18T20:14:43.911"}</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
@@ -10659,7 +10659,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":3,"count":2300022,"elapsedMs":378},"traceId":"10f1789d5e3841adac77a9c3ceb6c8b7","timestamp":"2026-08-18T09:50:47.212"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":3,"count":6,"elapsedMs":22},"traceId":"4c86b3408abc4ecbab25d791c904c584","timestamp":"2026-08-18T20:14:44.143"}</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr"/>
@@ -10692,7 +10692,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":0,"count":2300022,"elapsedMs":342},"traceId":"b0511b608ebf4ff8a12ece1472bcf075","timestamp":"2026-08-18T09:50:48.071"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":0,"count":6,"elapsedMs":3},"traceId":"ef65445f4873445baefa1050267eab1e","timestamp":"2026-08-18T20:14:44.363"}</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr"/>
@@ -10725,7 +10725,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求参数类型错误","data":null,"traceId":"29ed933ff0614380b4c9850514d9ea99","timestamp":"2026-08-18T09:50:48.304"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求参数类型错误","data":null,"traceId":"4f18218b1d5d47a7b3c5f7290f217833","timestamp":"2026-08-18T20:14:44.58"}</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
@@ -10758,7 +10758,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>PKXN][Content_Types].xml�S�n�0����*6�PU�C���\{�X�%����]8�R� q�cfgfW�d�q�ZCB|��|�*�*h㻆},^�{Va�^K&lt;4�6�N�XQ�ǆ�9�!P��$��҆�d�c�D�j);��ѝP�g��E�M'O�ʕ����H7L�h���R���G��^�'�{��zސʮB��3�˙��h.�h�W�жF�j娄C …</t>
+          <t>PK֡][Content_Types].xml�S�n�0����*6�PU�C���\{�X�%����]8�R� q�cfgfW�d�q�ZCB|��|�*�*h㻆},^�{Va�^K&lt;4�6�N�XQ�ǆ�9�!P��$��҆�d�c�D�j);��ѝP�g��E�M'O�ʕ����H7L�h���R���G��^�'�{��zސʮB��3�˙��h.�h�W�жF�j娄CQ …</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -10795,7 +10795,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"bb710d51fd834e2b880bbf6c0eefa695","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"7e65607843664536be93509c50a0f06d","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr"/>
@@ -10828,7 +10828,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"bb710d51fd834e2b880bbf6c0eefa695","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"totalCount":3,"completedCount":3,"retryCount":0,"maxRetryCount":3,"errorMe …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"7e65607843664536be93509c50a0f06d","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"totalCount":3,"completedCount":3,"retryCount":0,"maxRetryCount":3,"errorMe …</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -10865,7 +10865,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入任务不存在","data":null,"traceId":"1ef67b909f2a4c2c8790466c3d87573b","timestamp":"2026-08-18T09:50:53.453"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入任务不存在","data":null,"traceId":"669448e9cc0f4bf7a9b8644167088046","timestamp":"2026-08-18T20:14:47.636"}</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr"/>
@@ -10898,7 +10898,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入错误明细文件不存在","data":null,"traceId":"ae7960ed59f34d2396d288647d9fc876","timestamp":"2026-08-18T09:50:53.661"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入错误明细文件不存在","data":null,"traceId":"1583eaf888eb4b3b981b49fcc92fa71a","timestamp":"2026-08-18T20:14:47.801"}</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
@@ -10931,7 +10931,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"cf6679483a7a4fe6bb326860e7b652d8","timestamp":"2026-08-18T09:50:53.856"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"26d8e5fe794a48fdb60cb2ad4b018586","timestamp":"2026-08-18T20:14:47.96"}</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr"/>
@@ -10964,7 +10964,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件不能为空","data":null,"traceId":"ae79dfad00a04163a8ba436dbb665362","timestamp":"2026-08-18T09:50:54.038"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件不能为空","data":null,"traceId":"943deb10ba404e76865a6fbdae32d5d7","timestamp":"2026-08-18T20:14:48.144"}</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr"/>
@@ -10997,7 +10997,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件格式错误，请上传 .xlsx 文件","data":null,"traceId":"0c758b49993d46a58534a19179881537","timestamp":"2026-08-18T09:50:54.277"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件格式错误，请上传 .xlsx 文件","data":null,"traceId":"3b136af7a005417bace0a3c0ebd524f9","timestamp":"2026-08-18T20:14:48.319"}</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -11034,7 +11034,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr"/>
@@ -11067,7 +11067,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"a77b0f4392714386bf94ed7e17908f61","canceled":true},"traceId":"84113fe782624895bf6616f87a965426","timestamp":"2026-08-18T09:50:55.027"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"b21e98c4d0574d0b899e3c017f513dc7","canceled":false},"traceId":"13e0238a791c42a0a2606ef3372a6d16","timestamp":"2026-08-18T20:14:49.019"}</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -11100,7 +11100,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","status":"FAILED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"total":3,"exported":3,"sheetCount":1,"retryCount":0,"maxRetryCount":3,"fil …</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -11137,7 +11137,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>{"timestamp":"2026-08-18T01:50:57.647+00:00","status":404,"error":"Not Found","path":"/api/excel/not-exist"}</t>
+          <t>{"timestamp":"2026-08-18T12:14:49.411+00:00","status":404,"error":"Not Found","path":"/api/excel/not-exist"}</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
@@ -11170,7 +11170,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"dc3944f6a2a34889b8dd06b2fcc9c6a7","timestamp":"2026-08-18T09:50:57.894"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"092f4e596d214e6796dbb52f798c4791","timestamp":"2026-08-18T20:14:49.619"}</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr"/>
@@ -11188,12 +11188,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>302</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>302</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -11201,14 +11201,10 @@
           <t>✅ PASS</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"导出任务尚未完成","data":null,"traceId":"5098f04395ea4776a8732ff42fb2443c","timestamp":"2026-08-18T09:50:58.096"}</t>
-        </is>
-      </c>
+      <c r="F20" s="5" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>导出任务状态=FAILED；SUCCESS 才应 302，FAILED/CANCELED/未完成应 409</t>
+          <t>导出任务状态=SUCCESS；SUCCESS 才应 302，FAILED/CANCELED/未完成应 409</t>
         </is>
       </c>
     </row>
@@ -11240,7 +11236,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"f643b97d4bf141eab6c2bfac8e43612e","timestamp":"2026-08-18T09:50:58.284"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"95d3c10519a1450b9097918dbee3704f","timestamp":"2026-08-18T20:14:50.392"}</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
@@ -11273,7 +11269,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":32,"pageNo":1,"pageSize":5,"records":[{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"59dcbfe6a79a4d …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":57,"pageNo":1,"pageSize":5,"records":[{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"16637b590d2f45 …</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
@@ -11306,7 +11302,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":32,"pageNo":1,"pageSize":20,"records":[{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"59dcbfe6a79a4 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":57,"pageNo":1,"pageSize":20,"records":[{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"16637b590d2f4 …</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr"/>
@@ -11339,7 +11335,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":32,"pageNo":1,"pageSize":100,"records":[{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"59dcbfe6a79a …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":57,"pageNo":1,"pageSize":100,"records":[{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"16637b590d2f …</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr"/>
@@ -11372,7 +11368,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskStatus.GARBAGE","data":null,"traceId":"88bca51dd90d4e9393ec8e0e71875ea0","timestamp":"2026-08-18T09:50:59.663"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskStatus.GARBAGE","data":null,"traceId":"ce1b455b798946a1ab90e382d3ba701d","timestamp":"2026-08-18T20:14:51.273"}</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -11409,7 +11405,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskType.GARBAGE","data":null,"traceId":"f1ffe2deae2e42038a516c36cc8813aa","timestamp":"2026-08-18T09:50:59.842"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskType.GARBAGE","data":null,"traceId":"161cba68e5aa4904a4c29caa0115bab5","timestamp":"2026-08-18T20:14:51.444"}</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -11446,7 +11442,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"59dcbfe6a79a4d758901c2dd62f53623","status":"FAILED","progress …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"16637b590d2f45b89aa5b6349efee057","status":"SUCCESS","progres …</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr"/>
@@ -11479,7 +11475,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"4401ae82539c4a6eb6a261ebb955187b","timestamp":"2026-08-18T09:51:00.227"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"d5a6190da847490c8902edd9bb384882","timestamp":"2026-08-18T20:14:51.85"}</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
@@ -11512,7 +11508,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"0df794a4ebd048dba72fc646e1e307ed","timestamp":"2026-08-18T09:51:00.428"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"fd069e28004946b0a20dda3691323e1f","timestamp":"2026-08-18T20:14:52.041"}</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
@@ -11545,7 +11541,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","canceled":false},"traceId":"058c2964ac5b45d7b8cda02956663050","timestamp":"2026-08-18T09:51:00.687"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ca142fb261eb4a13894adee9cc678591","canceled":false},"traceId":"bcfec77bb378458bb4f2e9d1596ce827","timestamp":"2026-08-18T20:14:52.212"}</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -11567,12 +11563,12 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>409</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>409</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -11582,12 +11578,12 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"634557ec1ddf47beb757d3ae9c0f9794","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"59dcbfe6a79a4d758901c2dd62f53623","status":"CREATED","progres …</t>
+          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"01cb9af9addc43c08210b35f4f345cee","timestamp":"2026-08-18T20:14:52.395"}</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>重试前任务状态=FAILED；FAILED/CANCELED/EXPIRED 应 200，其余应 409</t>
+          <t>重试前任务状态=SUCCESS；FAILED/CANCELED/EXPIRED 应 200，其余应 409</t>
         </is>
       </c>
     </row>
@@ -11619,7 +11615,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"2a6d3fc5caec4aa181432be5e4d9ed93","timestamp":"2026-08-18T09:51:01.184"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"a39fcb07d75f47b0b4353fde55cd74e6","timestamp":"2026-08-18T20:14:52.584"}</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr"/>
@@ -11637,12 +11633,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>409</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>409</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -11652,12 +11648,12 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"a77b0f4392714386bf94ed7e17908f61","ownerId":"admin","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"0c86e89a083f4beba6c6ef4dc66ddcd6","status":"CREATED","progress …</t>
+          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"ebd5357c3b8a464698829a2da88a2e59","timestamp":"2026-08-18T20:14:52.978"}</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>重试前任务状态=CANCELED；空库或小数据量下取消可能来晚，若已 SUCCESS 则 409 为正确行为</t>
+          <t>重试前任务状态=SUCCESS；空库或小数据量下取消可能来晚，若已 SUCCESS 则 409 为正确行为</t>
         </is>
       </c>
     </row>
@@ -11689,7 +11685,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"c8baaec8b27b4ab59d32531dc7a8ec41","ownerId":"user-1","runControlCode":"RT87017861","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"a2fe161ab69d4e08bd7126616bf6b6f0","ownerId":"user-1","runControlCode":"RT87055292","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr"/>
@@ -11722,7 +11718,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码不能为空","data":null,"traceId":"3d31e5dbde4a445db581798d3d9ce797","timestamp":"2026-08-18T09:51:02.125"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码不能为空","data":null,"traceId":"00c55c58790c4893b17931f1ce67388f","timestamp":"2026-08-18T20:14:53.465"}</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr"/>
@@ -11755,7 +11751,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码已存在","data":null,"traceId":"138c828be7004621bf0249240fdd6893","timestamp":"2026-08-18T09:51:02.319"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码已存在","data":null,"traceId":"846bb56c5cac42a9892ad4bddc6b1dcd","timestamp":"2026-08-18T20:14:53.688"}</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr"/>
@@ -11788,7 +11784,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄必须在0到150之间","data":null,"traceId":"6c3965f2605f4656b1e4eb115dbb31b8","timestamp":"2026-08-18T09:51:02.528"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄必须在0到150之间","data":null,"traceId":"96258ae3787d4e2c97976d9cc316a23d","timestamp":"2026-08-18T20:14:53.867"}</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr"/>
@@ -11821,7 +11817,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最大年龄必须在0到150之间","data":null,"traceId":"fa793155b2a34db5b4131747b0ffddf6","timestamp":"2026-08-18T09:51:02.761"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最大年龄必须在0到150之间","data":null,"traceId":"710ccf6812f24b279ce79125b32b1857","timestamp":"2026-08-18T20:14:54.078"}</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
@@ -11854,7 +11850,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"836c24f810fd4bcb9e260dc020fc7dcb","timestamp":"2026-08-18T09:51:03.016"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"be31d414a2cb4ae48c45e030d59f6968","timestamp":"2026-08-18T20:14:54.283"}</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr"/>
@@ -11887,7 +11883,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"runId":"c8baaec8b27b4ab59d32531dc7a8ec41","ownerId":"user-1","runControlCode":"RT87017861","runName":"2026春季测试","studentNo":"T202608 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"runId":"a2fe161ab69d4e08bd7126616bf6b6f0","ownerId":"user-1","runControlCode":"RT87055292","runName":"2026春季测试","studentNo":"T202608 …</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr"/>
@@ -11920,7 +11916,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.excel.domain.model.StudentReportRunStatus.GARBAGE","data":null,"traceId":"ae1dbacd908b449bb19ce1f04bb895b9","timestamp":"2026-08-18T09:51:03.462"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.excel.domain.model.StudentReportRunStatus.GARBAGE","data":null,"traceId":"4add3da10f1d4f55bc3fd1b3438a180b","timestamp":"2026-08-18T20:14:54.684"}</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -11957,7 +11953,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"c8baaec8b27b4ab59d32531dc7a8ec41","ownerId":"user-1","runControlCode":"RT87017861","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"a2fe161ab69d4e08bd7126616bf6b6f0","ownerId":"user-1","runControlCode":"RT87055292","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
@@ -11990,7 +11986,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"804ef8dbb176422d9c658036963f7767","timestamp":"2026-08-18T09:51:03.909"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"feaf0cd1647344edb1b34041c7118f9d","timestamp":"2026-08-18T20:14:55.087"}</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr"/>
@@ -12023,7 +12019,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"f8a86b57aed745b280ce44858f556d61","timestamp":"2026-08-18T09:51:04.1"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"9786bb7682c248fa91a15c86d5660f9c","timestamp":"2026-08-18T20:14:55.275"}</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr"/>
@@ -12056,7 +12052,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"c8baaec8b27b4ab59d32531dc7a8ec41","ownerId":"user-1","runControlCode":"RT87017861","runName":"2026春季改","studentNo":null,"nameKeyword":null,"className":"一班","gender":null, …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"a2fe161ab69d4e08bd7126616bf6b6f0","ownerId":"user-1","runControlCode":"RT87055292","runName":"2026春季改","studentNo":null,"nameKeyword":null,"className":"一班","gender":null, …</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr"/>
@@ -12089,7 +12085,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"fe8382a2f7574814a1599fd20c537b26","timestamp":"2026-08-18T09:51:04.49"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"48badd33bdc34e3c9b56fb6533202ab5","timestamp":"2026-08-18T20:14:55.65"}</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr"/>
@@ -12122,7 +12118,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"7c058027f41a4b7984ed0856d1c5b065","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"1294e03bbfbe43d8a84abac8b59e4ff9","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr"/>
@@ -12155,7 +12151,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"taskId":"7c058027f41a4b7984ed0856d1c5b065","ownerId":"user-1","taskType":"EXPORT","taskName":"学生报表导出-2026春季改","businessKey":"c8baaec …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"taskId":"1294e03bbfbe43d8a84abac8b59e4ff9","ownerId":"user-1","taskType":"EXPORT","taskName":"学生报表导出-2026春季改","businessKey":"a2fe161 …</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr"/>
@@ -12188,7 +12184,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"c8baaec8b27b4ab59d32531dc7a8ec41","deleted":true},"traceId":"0ba044c2ad474632a9028b594e6f45cb","timestamp":"2026-08-18T09:51:05.978"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"a2fe161ab69d4e08bd7126616bf6b6f0","deleted":true},"traceId":"3f301bab77894caba6f1ba9837537775","timestamp":"2026-08-18T20:14:56.251"}</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr"/>
@@ -12221,7 +12217,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"57f4cb73a7964ca4898e256b6cc26cf6","timestamp":"2026-08-18T09:51:06.163"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"9c5d7e38c8bf411a820f9278f2774900","timestamp":"2026-08-18T20:14:56.42"}</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr"/>
@@ -12254,7 +12250,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"1bbf7dd099874d3698f4f6ada1e595f2","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fileExt":"txt","statu …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"cc8657c948024f158d1c3eab05dcda8c","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fileExt":"txt","statu …</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr"/>
@@ -12287,7 +12283,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"36f427f4ce53474f97e0badcc3caf959","timestamp":"2026-08-18T09:51:06.547"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"4c31bdad393c4057809bfa6e50a3f588","timestamp":"2026-08-18T20:14:56.803"}</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr"/>
@@ -12320,7 +12316,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"上传文件不能为空","data":null,"traceId":"9e35522f393848a6bc32ed7adeb724b2","timestamp":"2026-08-18T09:51:06.739"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"上传文件不能为空","data":null,"traceId":"a4aca0b143b649b1af2fd08ee1e71303","timestamp":"2026-08-18T20:14:56.988"}</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr"/>
@@ -12353,12 +12349,12 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件内容疑似可执行程序，originalName=evil.xlsx","data":null,"traceId":"4408cfb28ea84198af6b63788c32afc4","timestamp":"2026-08-18T09:51:06.957"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件内容疑似可执行程序，originalName=evil.xlsx","data":null,"traceId":"1284953fee1b4274b1ffd8cf58d6c6f6","timestamp":"2026-08-18T20:14:57.191"}</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>文件安全扫描：内容嗅探拦截伪装可执行文件 ✅</t>
+          <t>文件安全扫描应在落库前拦截伪装可执行内容</t>
         </is>
       </c>
     </row>
@@ -12390,7 +12386,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":true,"file":{"fileId":"1bbf7dd099874d3698f4f6ada1e595f2","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":true,"file":{"fileId":"cc8657c948024f158d1c3eab05dcda8c","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d …</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr"/>
@@ -12423,7 +12419,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":false,"file":null},"traceId":"1ad5344e60644569a8304d74f55b87a5","timestamp":"2026-08-18T09:51:07.491"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":false,"file":null},"traceId":"97adb1e4f36d4ebca41c3c3fe7589c72","timestamp":"2026-08-18T20:14:57.559"}</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr"/>
@@ -12456,7 +12452,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 不能为空","data":null,"traceId":"6a46098c28b94cfba78660dc5b40862f","timestamp":"2026-08-18T09:51:07.727"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 不能为空","data":null,"traceId":"ed6818ee39984333b0b0110037991d08","timestamp":"2026-08-18T20:14:57.744"}</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr"/>
@@ -12489,7 +12485,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"55e12b30dcbb462ba44719c36a043bdf","timestamp":"2026-08-18T09:51:07.947"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"340e2a61281046b7be0bb1270cba5c70","timestamp":"2026-08-18T20:14:57.9"}</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr"/>
@@ -12522,7 +12518,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件大小必须大于 0","data":null,"traceId":"c7a177741ba8495da784002f496c9cdc","timestamp":"2026-08-18T09:51:08.233"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件大小必须大于 0","data":null,"traceId":"49dd23fe4baa46b599aa4853196fb547","timestamp":"2026-08-18T20:14:58.073"}</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr"/>
@@ -12555,7 +12551,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"1bbf7dd099874d3698f4f6ada1e595f2","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fi …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"cc8657c948024f158d1c3eab05dcda8c","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fi …</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr"/>
@@ -12588,7 +12584,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"557d7598ef5b49df967243322a8f45f9","timestamp":"2026-08-18T09:51:08.653"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"86b5aa661d1142e593838a5c68e02f37","timestamp":"2026-08-18T20:14:58.467"}</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr"/>
@@ -12621,7 +12617,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":8,"pageNo":1,"pageSize":5,"records":[{"fileId":"1bbf7dd099874d3698f4f6ada1e595f2","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"f …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":13,"pageNo":1,"pageSize":5,"records":[{"fileId":"cc8657c948024f158d1c3eab05dcda8c","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223," …</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr"/>
@@ -12683,7 +12679,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"ce1509874776456a94cc064cef119a15","timestamp":"2026-08-18T09:51:09.637"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"81de94315809496b8aaa988356d8e631","timestamp":"2026-08-18T20:14:58.988"}</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr"/>
@@ -12716,7 +12712,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":true,"uploadId":null,"fileId":"1bbf7dd099874d3698f4f6ada1e595f2","uploadUrl":null,"objectKey":null,"expireMinutes":null,"file":{"fileId":"1bbf7dd099874d3698f4f6ada1e595f …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":true,"uploadId":null,"fileId":"cc8657c948024f158d1c3eab05dcda8c","uploadUrl":null,"objectKey":null,"expireMinutes":null,"file":{"fileId":"cc8657c948024f158d1c3eab05dcda8 …</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr"/>
@@ -12749,7 +12745,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"2ba416c64658459a8600e8a0fab4ddbd","timestamp":"2026-08-18T09:51:10.132"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"cbdc65e0ec45402f9fd600eff350a458","timestamp":"2026-08-18T20:14:59.349"}</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr"/>
@@ -12782,7 +12778,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"050c1f700349417fb8fd277cebc6101c","timestamp":"2026-08-18T09:51:10.416"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"6314dadc618c4cfca14fed6685c07c70","timestamp":"2026-08-18T20:14:59.548"}</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr"/>
@@ -12815,7 +12811,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"7830734486bf4a25bb95170d6438b887","fileId":"a834328e39ac41b6b10660af4c826bea","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"95be93177d6544e0ad0ae8542013a329","fileId":"785f8e1b0a2440218a8f1dd853fa9130","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr"/>
@@ -12848,7 +12844,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"uploadId":"7830734486bf4a25bb95170d6438b887","partCount":3,"uploadedParts":[1,2]},"traceId":"940bb22c851441d6be88f4d8c4974c56","timestamp":"2026-08-18T09:52:14.888"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"uploadId":"95be93177d6544e0ad0ae8542013a329","partCount":3,"uploadedParts":[1,2]},"traceId":"2f53a1225d384452846a1b9fa7f0b557","timestamp":"2026-08-18T20:15:10.192"}</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
@@ -12885,7 +12881,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"a834328e39ac41b6b10660af4c826bea","ownerId":"user-1","originalName":"big.bin","contentType":null,"fileSize":12582912,"fileMd5":"825b98cb69356d962a9006a51cbbadff","fileEx …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"785f8e1b0a2440218a8f1dd853fa9130","ownerId":"user-1","originalName":"big.bin","contentType":null,"fileSize":12582912,"fileMd5":"10257c05db7e818b1608140ef8b9fb4f","fileEx …</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr"/>
@@ -12918,7 +12914,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"bcb7b2d8c0a74001ba0b182014897d89","timestamp":"2026-08-18T09:52:29.379"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"7b85abbc0db7472998f743c040c05c1d","timestamp":"2026-08-18T20:15:12.896"}</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr"/>
@@ -12951,7 +12947,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"d6dc0c4cc5bb4cfcb82edd8c8d86d930","fileId":"ff0ff84b51a0474584cd5ce193e646f8","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"607cc187fe9047fdbe785938360a9efc","fileId":"427ec9fb7fd74ad38937ef9bfe0f85f6","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr"/>
@@ -12984,7 +12980,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"d6dc0c4cc5bb4cfcb82edd8c8d86d930"},"traceId":"abecf29242a74399b62f2800997359fd","timestamp":"2026-08-18T09:52:31.417"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"607cc187fe9047fdbe785938360a9efc"},"traceId":"33201486cfbd40ef91f643aef3a1a534","timestamp":"2026-08-18T20:15:13.39"}</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr"/>
@@ -13017,7 +13013,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"上传任务状态不允许完成，status=ABORTED","data":null,"traceId":"ec5651fe434e41daab45623b2dc2b2c9","timestamp":"2026-08-18T09:52:31.891"}</t>
+          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"上传任务状态不允许完成，status=ABORTED","data":null,"traceId":"abd794f4aa354e6cb09075a00fc358d6","timestamp":"2026-08-18T20:15:13.637"}</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr"/>
@@ -13050,7 +13046,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"2716cc045d824c0382552132c424e617","timestamp":"2026-08-18T09:52:32.24"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"c029a48ea6a846e3bdbc3960d59176a1","timestamp":"2026-08-18T20:15:13.902"}</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr"/>
@@ -13083,7 +13079,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"deleted":true,"fileId":"1bbf7dd099874d3698f4f6ada1e595f2"},"traceId":"d2fa48feab8c4aa88f3debc2e6184aaa","timestamp":"2026-08-18T09:52:32.7"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"deleted":true,"fileId":"cc8657c948024f158d1c3eab05dcda8c"},"traceId":"7c821a5175fc4c13acd1e6b806c469ec","timestamp":"2026-08-18T20:15:14.245"}</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr"/>
@@ -13116,7 +13112,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"7ea8fef722e947209bedfd5a739c0676","timestamp":"2026-08-18T09:52:33.033"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"63c9ae87009049369fa9bd6683d5ef3a","timestamp":"2026-08-18T20:15:14.523"}</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr"/>
@@ -13149,7 +13145,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"b355268fe94f4f6f9de3233af816b36a","timestamp":"2026-08-18T09:52:33.582"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"67208ad14fa5410e812c27da6f215270","timestamp":"2026-08-18T20:15:14.841"}</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr"/>
@@ -13162,7 +13158,7 @@
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>标准环境 R11（文件安全扫描版，2026-08-18 09:52）：总 77  ✅PASS 77  ❌FAIL 0 —— 含新增 FIL-UP-04 安全用例</t>
+          <t>标准环境 R14（F-13 修复版，2026-08-18 20:15）：总 77  ✅PASS 77  ❌FAIL 0 —— F-13 关闭，全部缺陷清零</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: strengthen async workflow reliability
</commit_message>
<xml_diff>
--- a/docs/test/接口扁平化测试用例.xlsx
+++ b/docs/test/接口扁平化测试用例.xlsx
@@ -9,12 +9,12 @@
   <sheets>
     <sheet name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="接口参数列表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="执行结果(标准环境R14)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="执行结果(标准环境R19)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$M$136</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'接口参数列表'!$A$1:$K$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'执行结果(标准环境R14)'!$A$1:$G$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'执行结果(标准环境R19)'!$A$1:$G$78</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7895,15 +7895,19 @@
       <c r="J122" s="5" t="inlineStr"/>
       <c r="K122" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>200</t>
         </is>
       </c>
       <c r="L122" s="5" t="inlineStr">
         <is>
-          <t>非 UPLOADING 抛 IllegalStateException</t>
-        </is>
-      </c>
-      <c r="M122" s="5" t="inlineStr"/>
+          <t>重复 abort 幂等（R19 起设计变更）：ABORTED 态返回 200 aborted=true；SUCCESS 态跳过</t>
+        </is>
+      </c>
+      <c r="M122" s="5" t="inlineStr">
+        <is>
+          <t>幂等重试安全</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -10589,7 +10593,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_UNAUTHORIZED","message":"请先登录","data":null,"traceId":"8c7234fa2d59431080dc1548e6e22beb","timestamp":"2026-08-18T20:14:43.744"}</t>
+          <t>{"success":false,"code":"COMMON_UNAUTHORIZED","message":"请先登录","data":null,"traceId":"0eb9beab6437456181ce8aa407a1165b","timestamp":"2026-08-21T11:02:50.906"}</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -10626,7 +10630,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"count":3},"traceId":"ca09c73c5a4245348c98e3c99f84041a","timestamp":"2026-08-18T20:14:43.911"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"count":3},"traceId":"a4f3508885c14919b489b24d95dfcadd","timestamp":"2026-08-21T11:02:51.177"}</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
@@ -10659,7 +10663,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":3,"count":6,"elapsedMs":22},"traceId":"4c86b3408abc4ecbab25d791c904c584","timestamp":"2026-08-18T20:14:44.143"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":3,"count":6,"elapsedMs":7},"traceId":"186c997ab343446b89ba1bd9608c7806","timestamp":"2026-08-21T11:02:51.485"}</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr"/>
@@ -10692,7 +10696,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":0,"count":6,"elapsedMs":3},"traceId":"ef65445f4873445baefa1050267eab1e","timestamp":"2026-08-18T20:14:44.363"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":0,"count":6,"elapsedMs":4},"traceId":"caa37d316b4749beb947b4afa6f37cb0","timestamp":"2026-08-21T11:02:51.742"}</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr"/>
@@ -10725,7 +10729,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求参数类型错误","data":null,"traceId":"4f18218b1d5d47a7b3c5f7290f217833","timestamp":"2026-08-18T20:14:44.58"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求参数类型错误","data":null,"traceId":"f767bd58b0bc4e9b9cc7123341204ca5","timestamp":"2026-08-21T11:02:51.96"}</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
@@ -10758,7 +10762,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>PK֡][Content_Types].xml�S�n�0����*6�PU�C���\{�X�%����]8�R� q�cfgfW�d�q�ZCB|��|�*�*h㻆},^�{Va�^K&lt;4�6�N�XQ�ǆ�9�!P��$��҆�d�c�D�j);��ѝP�g��E�M'O�ʕ����H7L�h���R���G��^�'�{��zސʮB��3�˙��h.�h�W�жF�j娄CQ …</t>
+          <t>PKZX][Content_Types].xml�S�n�0����*6�PU�C���\{�X�%����]8�R� q�cfgfW�d�q�ZCB|��|�*�*h㻆},^�{Va�^K&lt;4�6�N�XQ�ǆ�9�!P��$��҆�d�c�D�j);��ѝP�g��E�M'O�ʕ����H7L�h���R���G��^�'�{��zސʮB��3�˙��h.�h�W�жF�j娄C …</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -10795,7 +10799,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"7e65607843664536be93509c50a0f06d","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"facc32028ba846a5872e76641033a555","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr"/>
@@ -10828,7 +10832,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"7e65607843664536be93509c50a0f06d","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"totalCount":3,"completedCount":3,"retryCount":0,"maxRetryCount":3,"errorMe …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"facc32028ba846a5872e76641033a555","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"totalCount":3,"completedCount":3,"retryCount":0,"maxRetryCount":3,"errorMe …</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -10865,7 +10869,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入任务不存在","data":null,"traceId":"669448e9cc0f4bf7a9b8644167088046","timestamp":"2026-08-18T20:14:47.636"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入任务不存在","data":null,"traceId":"0864dbbc72ff49dfad10676ee259062d","timestamp":"2026-08-21T11:02:55.259"}</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr"/>
@@ -10898,7 +10902,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入错误明细文件不存在","data":null,"traceId":"1583eaf888eb4b3b981b49fcc92fa71a","timestamp":"2026-08-18T20:14:47.801"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入错误明细文件不存在","data":null,"traceId":"299cad4d3c0a4213997b53d7ce754805","timestamp":"2026-08-21T11:02:55.517"}</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
@@ -10931,7 +10935,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"26d8e5fe794a48fdb60cb2ad4b018586","timestamp":"2026-08-18T20:14:47.96"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"a4605891e0d041cc8cd3ebaf36fd44f0","timestamp":"2026-08-21T11:02:55.891"}</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr"/>
@@ -10964,7 +10968,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件不能为空","data":null,"traceId":"943deb10ba404e76865a6fbdae32d5d7","timestamp":"2026-08-18T20:14:48.144"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件不能为空","data":null,"traceId":"98c1453011e54471a27d5d241fb50da4","timestamp":"2026-08-21T11:02:56.174"}</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr"/>
@@ -10997,7 +11001,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件格式错误，请上传 .xlsx 文件","data":null,"traceId":"3b136af7a005417bace0a3c0ebd524f9","timestamp":"2026-08-18T20:14:48.319"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件格式错误，请上传 .xlsx 文件","data":null,"traceId":"de4315bd9a964188bf21b10036d66dfb","timestamp":"2026-08-21T11:02:56.449"}</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -11034,7 +11038,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr"/>
@@ -11067,7 +11071,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"b21e98c4d0574d0b899e3c017f513dc7","canceled":false},"traceId":"13e0238a791c42a0a2606ef3372a6d16","timestamp":"2026-08-18T20:14:49.019"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"8e8eebdd13804bfa962975dd7c0bcfae","canceled":false},"traceId":"95822c0bfab24af395e1c1bf91ee6e2b","timestamp":"2026-08-21T11:02:57.166"}</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -11100,7 +11104,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"total":3,"exported":3,"sheetCount":1,"retryCount":0,"maxRetryCount":3,"fil …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"total":3,"exported":3,"sheetCount":1,"retryCount":0,"maxRetryCount":3,"fil …</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -11137,7 +11141,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>{"timestamp":"2026-08-18T12:14:49.411+00:00","status":404,"error":"Not Found","path":"/api/excel/not-exist"}</t>
+          <t>{"timestamp":"2026-08-21T03:02:57.590+00:00","status":404,"error":"Not Found","path":"/api/excel/not-exist"}</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
@@ -11170,7 +11174,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"092f4e596d214e6796dbb52f798c4791","timestamp":"2026-08-18T20:14:49.619"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"b68991c6189e414f90b65865c58ab4da","timestamp":"2026-08-21T11:02:57.807"}</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr"/>
@@ -11236,7 +11240,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"95d3c10519a1450b9097918dbee3704f","timestamp":"2026-08-18T20:14:50.392"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"472cf11e6fd8420284fe1247d484ba72","timestamp":"2026-08-21T11:02:58.179"}</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
@@ -11269,7 +11273,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":57,"pageNo":1,"pageSize":5,"records":[{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"16637b590d2f45 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":83,"pageNo":1,"pageSize":5,"records":[{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"6ffc4f9026794e …</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
@@ -11302,7 +11306,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":57,"pageNo":1,"pageSize":20,"records":[{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"16637b590d2f4 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":83,"pageNo":1,"pageSize":20,"records":[{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"6ffc4f9026794 …</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr"/>
@@ -11335,7 +11339,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":57,"pageNo":1,"pageSize":100,"records":[{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"16637b590d2f …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":83,"pageNo":1,"pageSize":100,"records":[{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"6ffc4f902679 …</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr"/>
@@ -11368,7 +11372,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskStatus.GARBAGE","data":null,"traceId":"ce1b455b798946a1ab90e382d3ba701d","timestamp":"2026-08-18T20:14:51.273"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskStatus.GARBAGE","data":null,"traceId":"485d24c522784dbcbb4a74b1ba11e2ab","timestamp":"2026-08-21T11:02:59.466"}</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -11405,7 +11409,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskType.GARBAGE","data":null,"traceId":"161cba68e5aa4904a4c29caa0115bab5","timestamp":"2026-08-18T20:14:51.444"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskType.GARBAGE","data":null,"traceId":"d8ae979ed96042fe9306cb44b1132942","timestamp":"2026-08-21T11:02:59.675"}</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -11442,7 +11446,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ca142fb261eb4a13894adee9cc678591","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"16637b590d2f45b89aa5b6349efee057","status":"SUCCESS","progres …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"6ffc4f9026794e1fb6ddb374474b9eb0","status":"SUCCESS","progres …</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr"/>
@@ -11475,7 +11479,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"d5a6190da847490c8902edd9bb384882","timestamp":"2026-08-18T20:14:51.85"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"d71fb9bf0896403ea3af21c70b21b375","timestamp":"2026-08-21T11:03:00.105"}</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
@@ -11508,7 +11512,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"fd069e28004946b0a20dda3691323e1f","timestamp":"2026-08-18T20:14:52.041"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"68e6ccdcd4284c7aa2e41c76960b1ccf","timestamp":"2026-08-21T11:03:00.386"}</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
@@ -11541,7 +11545,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ca142fb261eb4a13894adee9cc678591","canceled":false},"traceId":"bcfec77bb378458bb4f2e9d1596ce827","timestamp":"2026-08-18T20:14:52.212"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","canceled":false},"traceId":"507e2ac8851b446ebf36039f0616448e","timestamp":"2026-08-21T11:03:00.649"}</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -11578,7 +11582,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"01cb9af9addc43c08210b35f4f345cee","timestamp":"2026-08-18T20:14:52.395"}</t>
+          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"8c445c09b95446848e9bd09c1ada28b0","timestamp":"2026-08-21T11:03:00.965"}</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
@@ -11615,7 +11619,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"a39fcb07d75f47b0b4353fde55cd74e6","timestamp":"2026-08-18T20:14:52.584"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"8969253677564bdd9ca782f013b8e74e","timestamp":"2026-08-21T11:03:01.208"}</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr"/>
@@ -11648,7 +11652,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"ebd5357c3b8a464698829a2da88a2e59","timestamp":"2026-08-18T20:14:52.978"}</t>
+          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"c051e7affc9f45079a1905f24065e81b","timestamp":"2026-08-21T11:03:01.691"}</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -11685,7 +11689,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"a2fe161ab69d4e08bd7126616bf6b6f0","ownerId":"user-1","runControlCode":"RT87055292","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"3fb1fb9ad06143c3b014b3445f34c7bf","ownerId":"user-1","runControlCode":"RT87281381","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr"/>
@@ -11718,7 +11722,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码不能为空","data":null,"traceId":"00c55c58790c4893b17931f1ce67388f","timestamp":"2026-08-18T20:14:53.465"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码不能为空","data":null,"traceId":"c1b2e228ba7d4e4d8668f2be06efe477","timestamp":"2026-08-21T11:03:02.095"}</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr"/>
@@ -11751,7 +11755,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码已存在","data":null,"traceId":"846bb56c5cac42a9892ad4bddc6b1dcd","timestamp":"2026-08-18T20:14:53.688"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码已存在","data":null,"traceId":"d08184383ab4475c8c3170347744d116","timestamp":"2026-08-21T11:03:02.566"}</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr"/>
@@ -11784,7 +11788,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄必须在0到150之间","data":null,"traceId":"96258ae3787d4e2c97976d9cc316a23d","timestamp":"2026-08-18T20:14:53.867"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄必须在0到150之间","data":null,"traceId":"f4e09697922942cc806d084263dce974","timestamp":"2026-08-21T11:03:03.09"}</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr"/>
@@ -11817,7 +11821,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最大年龄必须在0到150之间","data":null,"traceId":"710ccf6812f24b279ce79125b32b1857","timestamp":"2026-08-18T20:14:54.078"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最大年龄必须在0到150之间","data":null,"traceId":"12c14df3770944a49ad9bbe35b3caf37","timestamp":"2026-08-21T11:03:03.387"}</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
@@ -11850,7 +11854,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"be31d414a2cb4ae48c45e030d59f6968","timestamp":"2026-08-18T20:14:54.283"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"a057f1ea0c284aab81d410f49340876b","timestamp":"2026-08-21T11:03:03.6"}</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr"/>
@@ -11883,7 +11887,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"runId":"a2fe161ab69d4e08bd7126616bf6b6f0","ownerId":"user-1","runControlCode":"RT87055292","runName":"2026春季测试","studentNo":"T202608 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"runId":"3fb1fb9ad06143c3b014b3445f34c7bf","ownerId":"user-1","runControlCode":"RT87281381","runName":"2026春季测试","studentNo":"T202608 …</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr"/>
@@ -11916,7 +11920,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.excel.domain.model.StudentReportRunStatus.GARBAGE","data":null,"traceId":"4add3da10f1d4f55bc3fd1b3438a180b","timestamp":"2026-08-18T20:14:54.684"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.excel.domain.model.StudentReportRunStatus.GARBAGE","data":null,"traceId":"1b741fc2536b417b9d0d22c821612bea","timestamp":"2026-08-21T11:03:04.144"}</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -11953,7 +11957,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"a2fe161ab69d4e08bd7126616bf6b6f0","ownerId":"user-1","runControlCode":"RT87055292","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"3fb1fb9ad06143c3b014b3445f34c7bf","ownerId":"user-1","runControlCode":"RT87281381","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
@@ -11986,7 +11990,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"feaf0cd1647344edb1b34041c7118f9d","timestamp":"2026-08-18T20:14:55.087"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"c572b82dab1f497c843ccf21d1c9d6f9","timestamp":"2026-08-21T11:03:04.676"}</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr"/>
@@ -12019,7 +12023,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"9786bb7682c248fa91a15c86d5660f9c","timestamp":"2026-08-18T20:14:55.275"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"221412809bb74347a50effe9bae941d7","timestamp":"2026-08-21T11:03:04.897"}</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr"/>
@@ -12052,7 +12056,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"a2fe161ab69d4e08bd7126616bf6b6f0","ownerId":"user-1","runControlCode":"RT87055292","runName":"2026春季改","studentNo":null,"nameKeyword":null,"className":"一班","gender":null, …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"3fb1fb9ad06143c3b014b3445f34c7bf","ownerId":"user-1","runControlCode":"RT87281381","runName":"2026春季改","studentNo":null,"nameKeyword":null,"className":"一班","gender":null, …</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr"/>
@@ -12085,7 +12089,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"48badd33bdc34e3c9b56fb6533202ab5","timestamp":"2026-08-18T20:14:55.65"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"26a52fd7ebbd431fb39e787e0bd6936a","timestamp":"2026-08-21T11:03:05.448"}</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr"/>
@@ -12118,7 +12122,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"1294e03bbfbe43d8a84abac8b59e4ff9","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"a447c0e34c8245dfaa2758373cf7ec4a","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr"/>
@@ -12151,7 +12155,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"taskId":"1294e03bbfbe43d8a84abac8b59e4ff9","ownerId":"user-1","taskType":"EXPORT","taskName":"学生报表导出-2026春季改","businessKey":"a2fe161 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"taskId":"a447c0e34c8245dfaa2758373cf7ec4a","ownerId":"user-1","taskType":"EXPORT","taskName":"学生报表导出-2026春季改","businessKey":"3fb1fb9 …</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr"/>
@@ -12184,7 +12188,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"a2fe161ab69d4e08bd7126616bf6b6f0","deleted":true},"traceId":"3f301bab77894caba6f1ba9837537775","timestamp":"2026-08-18T20:14:56.251"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"3fb1fb9ad06143c3b014b3445f34c7bf","deleted":true},"traceId":"f5beb3e7b9b34aa88f524de5c7048ec3","timestamp":"2026-08-21T11:03:06.21"}</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr"/>
@@ -12217,7 +12221,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"9c5d7e38c8bf411a820f9278f2774900","timestamp":"2026-08-18T20:14:56.42"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"00f9bce3f4ef4cd688de63163f971870","timestamp":"2026-08-21T11:03:06.455"}</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr"/>
@@ -12250,7 +12254,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"cc8657c948024f158d1c3eab05dcda8c","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fileExt":"txt","statu …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"0d4da69927cc4718b1576c7ce5a6650f","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fileExt":"txt","statu …</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr"/>
@@ -12283,7 +12287,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"4c31bdad393c4057809bfa6e50a3f588","timestamp":"2026-08-18T20:14:56.803"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"4937e8ee6f3640409fcfb65c9a2a5689","timestamp":"2026-08-21T11:03:06.893"}</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr"/>
@@ -12316,7 +12320,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"上传文件不能为空","data":null,"traceId":"a4aca0b143b649b1af2fd08ee1e71303","timestamp":"2026-08-18T20:14:56.988"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"上传文件不能为空","data":null,"traceId":"541218480d88486abc6f085a5600b218","timestamp":"2026-08-21T11:03:07.155"}</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr"/>
@@ -12349,7 +12353,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件内容疑似可执行程序，originalName=evil.xlsx","data":null,"traceId":"1284953fee1b4274b1ffd8cf58d6c6f6","timestamp":"2026-08-18T20:14:57.191"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件内容疑似可执行程序，originalName=evil.xlsx","data":null,"traceId":"46cd4c5be2ae41ca83d502cb45920557","timestamp":"2026-08-21T11:03:07.531"}</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -12386,7 +12390,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":true,"file":{"fileId":"cc8657c948024f158d1c3eab05dcda8c","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":true,"file":{"fileId":"0d4da69927cc4718b1576c7ce5a6650f","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d …</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr"/>
@@ -12419,7 +12423,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":false,"file":null},"traceId":"97adb1e4f36d4ebca41c3c3fe7589c72","timestamp":"2026-08-18T20:14:57.559"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":false,"file":null},"traceId":"758729c6386a424b876472894e3c1d55","timestamp":"2026-08-21T11:03:08.061"}</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr"/>
@@ -12452,7 +12456,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 不能为空","data":null,"traceId":"ed6818ee39984333b0b0110037991d08","timestamp":"2026-08-18T20:14:57.744"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 不能为空","data":null,"traceId":"5b0c193399dd44be824e20ffaad09e0c","timestamp":"2026-08-21T11:03:08.321"}</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr"/>
@@ -12485,7 +12489,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"340e2a61281046b7be0bb1270cba5c70","timestamp":"2026-08-18T20:14:57.9"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"8afce5ad38ff45439f82b61249b67e68","timestamp":"2026-08-21T11:03:08.537"}</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr"/>
@@ -12518,7 +12522,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件大小必须大于 0","data":null,"traceId":"49dd23fe4baa46b599aa4853196fb547","timestamp":"2026-08-18T20:14:58.073"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件大小必须大于 0","data":null,"traceId":"53da59adbe8d4552b2d206e126f4d060","timestamp":"2026-08-21T11:03:08.743"}</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr"/>
@@ -12551,7 +12555,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"cc8657c948024f158d1c3eab05dcda8c","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fi …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"0d4da69927cc4718b1576c7ce5a6650f","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fi …</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr"/>
@@ -12584,7 +12588,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"86b5aa661d1142e593838a5c68e02f37","timestamp":"2026-08-18T20:14:58.467"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"6d8dfb1960f24e26908fcb2d4f49f2e1","timestamp":"2026-08-21T11:03:09.161"}</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr"/>
@@ -12617,7 +12621,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":13,"pageNo":1,"pageSize":5,"records":[{"fileId":"cc8657c948024f158d1c3eab05dcda8c","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":25,"pageNo":1,"pageSize":5,"records":[{"fileId":"0d4da69927cc4718b1576c7ce5a6650f","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223," …</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr"/>
@@ -12679,7 +12683,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"81de94315809496b8aaa988356d8e631","timestamp":"2026-08-18T20:14:58.988"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"ef2acce117e14cf9aea00b1971b7eb28","timestamp":"2026-08-21T11:03:09.85"}</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr"/>
@@ -12712,7 +12716,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":true,"uploadId":null,"fileId":"cc8657c948024f158d1c3eab05dcda8c","uploadUrl":null,"objectKey":null,"expireMinutes":null,"file":{"fileId":"cc8657c948024f158d1c3eab05dcda8 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":true,"uploadId":null,"fileId":"0d4da69927cc4718b1576c7ce5a6650f","uploadUrl":null,"objectKey":null,"expireMinutes":null,"file":{"fileId":"0d4da69927cc4718b1576c7ce5a6650 …</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr"/>
@@ -12745,7 +12749,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"cbdc65e0ec45402f9fd600eff350a458","timestamp":"2026-08-18T20:14:59.349"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"e9343db0b1c6486ebab085c61e9fe3f7","timestamp":"2026-08-21T11:03:10.265"}</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr"/>
@@ -12778,7 +12782,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"6314dadc618c4cfca14fed6685c07c70","timestamp":"2026-08-18T20:14:59.548"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"88cde7f247314db09902787ade2bec80","timestamp":"2026-08-21T11:03:10.452"}</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr"/>
@@ -12811,7 +12815,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"95be93177d6544e0ad0ae8542013a329","fileId":"785f8e1b0a2440218a8f1dd853fa9130","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"185665793a26433ab621915d71f9efe2","fileId":"32e4d4e697334041a079f5c290e08234","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr"/>
@@ -12844,7 +12848,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"uploadId":"95be93177d6544e0ad0ae8542013a329","partCount":3,"uploadedParts":[1,2]},"traceId":"2f53a1225d384452846a1b9fa7f0b557","timestamp":"2026-08-18T20:15:10.192"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"uploadId":"185665793a26433ab621915d71f9efe2","partCount":3,"uploadedParts":[1,2]},"traceId":"56448cdbbbaa48048a143874ba8350b8","timestamp":"2026-08-21T11:04:34.362"}</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
@@ -12881,7 +12885,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"785f8e1b0a2440218a8f1dd853fa9130","ownerId":"user-1","originalName":"big.bin","contentType":null,"fileSize":12582912,"fileMd5":"10257c05db7e818b1608140ef8b9fb4f","fileEx …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"32e4d4e697334041a079f5c290e08234","ownerId":"user-1","originalName":"big.bin","contentType":null,"fileSize":12582912,"fileMd5":"d4f79b4066eeab2fdd4ffeb11e211d19","fileEx …</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr"/>
@@ -12914,7 +12918,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"7b85abbc0db7472998f743c040c05c1d","timestamp":"2026-08-18T20:15:12.896"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"cf2e15d648c749c2a569082bedcb4ac9","timestamp":"2026-08-21T11:04:54.676"}</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr"/>
@@ -12947,7 +12951,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"607cc187fe9047fdbe785938360a9efc","fileId":"427ec9fb7fd74ad38937ef9bfe0f85f6","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"9e9e2100e2aa4eaebe2486b32c3faf17","fileId":"3548569735114270b676862dd622e0bf","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr"/>
@@ -12980,7 +12984,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"607cc187fe9047fdbe785938360a9efc"},"traceId":"33201486cfbd40ef91f643aef3a1a534","timestamp":"2026-08-18T20:15:13.39"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"9e9e2100e2aa4eaebe2486b32c3faf17"},"traceId":"55f29f6eb55d4a52a75c1464fbdcf06e","timestamp":"2026-08-21T11:04:55.731"}</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr"/>
@@ -12998,12 +13002,12 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
@@ -13013,10 +13017,14 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"上传任务状态不允许完成，status=ABORTED","data":null,"traceId":"abd794f4aa354e6cb09075a00fc358d6","timestamp":"2026-08-18T20:15:13.637"}</t>
-        </is>
-      </c>
-      <c r="G74" s="5" t="inlineStr"/>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"9e9e2100e2aa4eaebe2486b32c3faf17"},"traceId":"d26345b164f142899f64aedd88e91aee","timestamp":"2026-08-21T11:04:56.105"}</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>R19 行为变更：重复 abort 幂等化（200）</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -13046,7 +13054,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"c029a48ea6a846e3bdbc3960d59176a1","timestamp":"2026-08-18T20:15:13.902"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"6d444a64d14040a89a15933d033f06dc","timestamp":"2026-08-21T11:04:56.654"}</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr"/>
@@ -13079,7 +13087,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"deleted":true,"fileId":"cc8657c948024f158d1c3eab05dcda8c"},"traceId":"7c821a5175fc4c13acd1e6b806c469ec","timestamp":"2026-08-18T20:15:14.245"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"deleted":true,"fileId":"0d4da69927cc4718b1576c7ce5a6650f"},"traceId":"2ffc3bcc02754502a44bffb7fee42032","timestamp":"2026-08-21T11:04:57.144"}</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr"/>
@@ -13112,7 +13120,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"63c9ae87009049369fa9bd6683d5ef3a","timestamp":"2026-08-18T20:15:14.523"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"a2f17b1b74254d2a82e867b2734d74c1","timestamp":"2026-08-21T11:04:57.387"}</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr"/>
@@ -13145,7 +13153,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"67208ad14fa5410e812c27da6f215270","timestamp":"2026-08-18T20:15:14.841"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"c7bb842f64b944c09dde47bac3a79ecf","timestamp":"2026-08-21T11:04:57.666"}</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr"/>
@@ -13158,7 +13166,7 @@
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>标准环境 R14（F-13 修复版，2026-08-18 20:15）：总 77  ✅PASS 77  ❌FAIL 0 —— F-13 关闭，全部缺陷清零</t>
+          <t>标准环境 R19（执行租约版，2026-08-21）：总 77  ✅PASS 77  ❌FAIL 0 —— task:execution 租约实测捕获；abort 幂等行为变更已同步用例；单测 104/104</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add auth and ops dashboard workflow
</commit_message>
<xml_diff>
--- a/docs/test/接口扁平化测试用例.xlsx
+++ b/docs/test/接口扁平化测试用例.xlsx
@@ -9,12 +9,12 @@
   <sheets>
     <sheet name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="接口参数列表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="执行结果(标准环境R19)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="执行结果(标准环境R22)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$M$136</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'接口参数列表'!$A$1:$K$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'执行结果(标准环境R19)'!$A$1:$G$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'执行结果(标准环境R22)'!$A$1:$G$78</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -10593,7 +10593,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_UNAUTHORIZED","message":"请先登录","data":null,"traceId":"0eb9beab6437456181ce8aa407a1165b","timestamp":"2026-08-21T11:02:50.906"}</t>
+          <t>{"success":false,"code":"SECURITY_UNAUTHORIZED","message":"请先登录","data":null,"traceId":"70162071950c448ba1057f12e4582bc4","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:04:57.972"}</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"count":3},"traceId":"a4f3508885c14919b489b24d95dfcadd","timestamp":"2026-08-21T11:02:51.177"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"count":3},"traceId":"1ccc82d3495e4e499904b52982929d84","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:04:58.198"}</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
@@ -10663,7 +10663,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":3,"count":6,"elapsedMs":7},"traceId":"186c997ab343446b89ba1bd9608c7806","timestamp":"2026-08-21T11:02:51.485"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":3,"count":6,"elapsedMs":7},"traceId":"a5484de817df4d08bc1ad6244bd33298","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:04 …</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr"/>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":0,"count":6,"elapsedMs":4},"traceId":"caa37d316b4749beb947b4afa6f37cb0","timestamp":"2026-08-21T11:02:51.742"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":0,"count":6,"elapsedMs":2},"traceId":"49a97b8292884130a42e8b689a897c6e","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:04 …</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr"/>
@@ -10729,7 +10729,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求参数类型错误","data":null,"traceId":"f767bd58b0bc4e9b9cc7123341204ca5","timestamp":"2026-08-21T11:02:51.96"}</t>
+          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"请求参数类型错误","data":null,"traceId":"fe3c86936320497fad9866cf676c7a0a","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:04:58.785"}</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
@@ -10762,7 +10762,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>PKZX][Content_Types].xml�S�n�0����*6�PU�C���\{�X�%����]8�R� q�cfgfW�d�q�ZCB|��|�*�*h㻆},^�{Va�^K&lt;4�6�N�XQ�ǆ�9�!P��$��҆�d�c�D�j);��ѝP�g��E�M'O�ʕ����H7L�h���R���G��^�'�{��zސʮB��3�˙��h.�h�W�жF�j娄C …</t>
+          <t>PK�P][Content_Types].xml�S�n�0����*6�PU�C���\{�X�%����]8�R� q�cfgfW�d�q�ZCB|��|�*�*h㻆},^�{Va�^K&lt;4�6�N�XQ�ǆ�9�!P��$��҆�d�c�D�j);��ѝP�g��E�M'O�ʕ����H7L�h���R���G��^�'�{��zސʮB��3�˙��h.�h�W�жF�j娄C …</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
@@ -10799,7 +10799,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"facc32028ba846a5872e76641033a555","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"d1bbb191375d403585ef7690f53db10b","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr"/>
@@ -10832,7 +10832,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"facc32028ba846a5872e76641033a555","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"totalCount":3,"completedCount":3,"retryCount":0,"maxRetryCount":3,"errorMe …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"d1bbb191375d403585ef7690f53db10b","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"totalCount":3,"completedCount":3,"retryCount":0,"maxRetryCount":3,"errorMe …</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -10869,7 +10869,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入任务不存在","data":null,"traceId":"0864dbbc72ff49dfad10676ee259062d","timestamp":"2026-08-21T11:02:55.259"}</t>
+          <t>{"success":false,"code":"EXCEL_TASK_NOT_FOUND","message":"导入任务不存在","data":null,"traceId":"ddd17c435ee54347927a86ea60ce6628","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:01.998"}</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr"/>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导入错误明细文件不存在","data":null,"traceId":"299cad4d3c0a4213997b53d7ce754805","timestamp":"2026-08-21T11:02:55.517"}</t>
+          <t>{"success":false,"code":"EXCEL_FILE_NOT_FOUND","message":"导入错误明细文件不存在","data":null,"traceId":"e53941234d7d44efbdcd7502e4e58ca0","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:02.246"}</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
@@ -10935,7 +10935,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"a4605891e0d041cc8cd3ebaf36fd44f0","timestamp":"2026-08-21T11:02:55.891"}</t>
+          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"b7bc32e656ef43cca8502f8308cdd668","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:02.469"}</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr"/>
@@ -10968,7 +10968,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件不能为空","data":null,"traceId":"98c1453011e54471a27d5d241fb50da4","timestamp":"2026-08-21T11:02:56.174"}</t>
+          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"导入文件不能为空","data":null,"traceId":"cf61812007ae415c876a923beab8c9d1","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:02.681"}</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr"/>
@@ -11001,7 +11001,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"导入文件格式错误，请上传 .xlsx 文件","data":null,"traceId":"de4315bd9a964188bf21b10036d66dfb","timestamp":"2026-08-21T11:02:56.449"}</t>
+          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"导入文件格式错误，请上传 .xlsx 文件","data":null,"traceId":"2dea2f57f7db49e9b19a6f5fc06ff546","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:02.844"}</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -11038,7 +11038,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr"/>
@@ -11071,7 +11071,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"8e8eebdd13804bfa962975dd7c0bcfae","canceled":false},"traceId":"95822c0bfab24af395e1c1bf91ee6e2b","timestamp":"2026-08-21T11:02:57.166"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"92345433cb134e98b86e527d034421e2","canceled":false},"traceId":"1566d9e58a494366b2f0110f4da5c98c","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -11104,7 +11104,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"total":3,"exported":3,"sheetCount":1,"retryCount":0,"maxRetryCount":3,"fil …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"total":3,"exported":3,"sheetCount":1,"retryCount":0,"maxRetryCount":3,"fil …</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -11141,7 +11141,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>{"timestamp":"2026-08-21T03:02:57.590+00:00","status":404,"error":"Not Found","path":"/api/excel/not-exist"}</t>
+          <t>{"timestamp":"2026-08-22T02:05:03.870+00:00","status":404,"error":"Not Found","path":"/api/excel/not-exist"}</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
@@ -11174,7 +11174,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"b68991c6189e414f90b65865c58ab4da","timestamp":"2026-08-21T11:02:57.807"}</t>
+          <t>{"success":false,"code":"EXCEL_TASK_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"7f86aa0e808d47b3b0fbf99da0f4253a","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:04.067"}</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr"/>
@@ -11240,7 +11240,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"472cf11e6fd8420284fe1247d484ba72","timestamp":"2026-08-21T11:02:58.179"}</t>
+          <t>{"success":false,"code":"EXCEL_TASK_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"b2505d41ca3b4784bd827625fd7270c7","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:04.438"}</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
@@ -11273,7 +11273,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":83,"pageNo":1,"pageSize":5,"records":[{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"6ffc4f9026794e …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":122,"pageNo":1,"pageSize":5,"records":[{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"b7ff83e8167a4 …</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
@@ -11306,7 +11306,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":83,"pageNo":1,"pageSize":20,"records":[{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"6ffc4f9026794 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":122,"pageNo":1,"pageSize":20,"records":[{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"b7ff83e8167a …</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr"/>
@@ -11324,12 +11324,12 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -11339,10 +11339,14 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":83,"pageNo":1,"pageSize":100,"records":[{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"6ffc4f902679 …</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr"/>
+          <t>{"success":false,"code":"TASK_PARAM_ERROR","message":"请求参数校验失败","data":null,"traceId":"2efab826a1fb4b349442d09a32ee336c","bizId":null,"retryable":false,"suggestion":"请根据 fieldErrors 修正请求参数","fieldErrors":[{"field":"pageSize","message":"每页条数 …</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>R22 行为变更：越界分页参数 400 拒绝（ERR-03 Bean Validation）</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -11372,7 +11376,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskStatus.GARBAGE","data":null,"traceId":"485d24c522784dbcbb4a74b1ba11e2ab","timestamp":"2026-08-21T11:02:59.466"}</t>
+          <t>{"success":false,"code":"TASK_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskStatus.GARBAGE","data":null,"traceId":"c2d53040642747b79a9631d263c73b04","bizId":null,"retryable":null,"suggestion":null,"field …</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -11409,7 +11413,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskType.GARBAGE","data":null,"traceId":"d8ae979ed96042fe9306cb44b1132942","timestamp":"2026-08-21T11:02:59.675"}</t>
+          <t>{"success":false,"code":"TASK_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskType.GARBAGE","data":null,"traceId":"21234cfefbc5416d95412d22bcd4aa14","bizId":null,"retryable":null,"suggestion":null,"fieldEr …</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -11446,7 +11450,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"6ffc4f9026794e1fb6ddb374474b9eb0","status":"SUCCESS","progres …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"b7ff83e8167a47b9a7989d218c2aee5d","status":"SUCCESS","progres …</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr"/>
@@ -11479,7 +11483,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"d71fb9bf0896403ea3af21c70b21b375","timestamp":"2026-08-21T11:03:00.105"}</t>
+          <t>{"success":false,"code":"TASK_NOT_FOUND","message":"任务不存在","data":null,"traceId":"c4001e13accb4ca497f1ead62eb0722e","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:06.188"}</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
@@ -11512,7 +11516,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"68e6ccdcd4284c7aa2e41c76960b1ccf","timestamp":"2026-08-21T11:03:00.386"}</t>
+          <t>{"success":false,"code":"TASK_NOT_FOUND","message":"任务不存在","data":null,"traceId":"5f69a0162109454e919d5856ab7c5fe3","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:06.381"}</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
@@ -11545,7 +11549,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"f8bc1b7f5d974e2c870e8e8654175070","canceled":false},"traceId":"507e2ac8851b446ebf36039f0616448e","timestamp":"2026-08-21T11:03:00.649"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","canceled":false},"traceId":"010d78d324934cc294347d8a23412936","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -11582,7 +11586,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"8c445c09b95446848e9bd09c1ada28b0","timestamp":"2026-08-21T11:03:00.965"}</t>
+          <t>{"success":false,"code":"TASK_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"fe9d046fdf3b49a8885f30145b3288e3","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:0 …</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
@@ -11619,7 +11623,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"任务不存在","data":null,"traceId":"8969253677564bdd9ca782f013b8e74e","timestamp":"2026-08-21T11:03:01.208"}</t>
+          <t>{"success":false,"code":"TASK_NOT_FOUND","message":"任务不存在","data":null,"traceId":"89985f5a6b1149399a0a251695eafc7b","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:07.184"}</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr"/>
@@ -11652,7 +11656,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"c051e7affc9f45079a1905f24065e81b","timestamp":"2026-08-21T11:03:01.691"}</t>
+          <t>{"success":false,"code":"TASK_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"3f0e8fb2a47f40f58f9d82dda8ef8c48","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:0 …</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -11689,7 +11693,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"3fb1fb9ad06143c3b014b3445f34c7bf","ownerId":"user-1","runControlCode":"RT87281381","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a9cd8db6838443eb747df8151b7c596","ownerId":"user-1","runControlCode":"RT87364303","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr"/>
@@ -11722,7 +11726,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码不能为空","data":null,"traceId":"c1b2e228ba7d4e4d8668f2be06efe477","timestamp":"2026-08-21T11:03:02.095"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码不能为空","data":null,"traceId":"783c68fa85724761b3e4d55d3078bc17","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:08.076"}</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr"/>
@@ -11755,7 +11759,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码已存在","data":null,"traceId":"d08184383ab4475c8c3170347744d116","timestamp":"2026-08-21T11:03:02.566"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码已存在","data":null,"traceId":"51809234343b48d6853d37d82f2d61f2","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:08.257"}</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr"/>
@@ -11788,7 +11792,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄必须在0到150之间","data":null,"traceId":"f4e09697922942cc806d084263dce974","timestamp":"2026-08-21T11:03:03.09"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄必须在0到150之间","data":null,"traceId":"33b30b25f95748f5b3da9bc850c27f10","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:08.456"}</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr"/>
@@ -11821,7 +11825,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最大年龄必须在0到150之间","data":null,"traceId":"12c14df3770944a49ad9bbe35b3caf37","timestamp":"2026-08-21T11:03:03.387"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最大年龄必须在0到150之间","data":null,"traceId":"8936f866a34943f4a5baabd453252adf","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:08.684"}</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
@@ -11854,7 +11858,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"a057f1ea0c284aab81d410f49340876b","timestamp":"2026-08-21T11:03:03.6"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"d61401405c1d4b09baffaf0bd21deea6","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:08.867"}</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr"/>
@@ -11887,7 +11891,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"runId":"3fb1fb9ad06143c3b014b3445f34c7bf","ownerId":"user-1","runControlCode":"RT87281381","runName":"2026春季测试","studentNo":"T202608 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"runId":"8a9cd8db6838443eb747df8151b7c596","ownerId":"user-1","runControlCode":"RT87364303","runName":"2026春季测试","studentNo":"T202608 …</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr"/>
@@ -11920,7 +11924,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.excel.domain.model.StudentReportRunStatus.GARBAGE","data":null,"traceId":"1b741fc2536b417b9d0d22c821612bea","timestamp":"2026-08-21T11:03:04.144"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.excel.domain.model.StudentReportRunStatus.GARBAGE","data":null,"traceId":"0340bae5d8354fe5bf2b5075dadc9075","bizId":null,"retryable":null,"suggestion":n …</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -11957,7 +11961,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"3fb1fb9ad06143c3b014b3445f34c7bf","ownerId":"user-1","runControlCode":"RT87281381","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a9cd8db6838443eb747df8151b7c596","ownerId":"user-1","runControlCode":"RT87364303","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
@@ -11990,7 +11994,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"c572b82dab1f497c843ccf21d1c9d6f9","timestamp":"2026-08-21T11:03:04.676"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"cd426004567f4067b9f19c4be3916762","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:09.672"}</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr"/>
@@ -12023,7 +12027,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"221412809bb74347a50effe9bae941d7","timestamp":"2026-08-21T11:03:04.897"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"dc2aadce2dec44a8b9f1320232f76e85","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:09.882"}</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr"/>
@@ -12056,7 +12060,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"3fb1fb9ad06143c3b014b3445f34c7bf","ownerId":"user-1","runControlCode":"RT87281381","runName":"2026春季改","studentNo":null,"nameKeyword":null,"className":"一班","gender":null, …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a9cd8db6838443eb747df8151b7c596","ownerId":"user-1","runControlCode":"RT87364303","runName":"2026春季改","studentNo":null,"nameKeyword":null,"className":"一班","gender":null, …</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr"/>
@@ -12089,7 +12093,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"26a52fd7ebbd431fb39e787e0bd6936a","timestamp":"2026-08-21T11:03:05.448"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"58a9f298a7dd4203b11ea8f55b4ab7a7","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:10.299"}</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr"/>
@@ -12122,7 +12126,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"a447c0e34c8245dfaa2758373cf7ec4a","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"e32cd8971e3343cb8cf979eaf0531e7a","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr"/>
@@ -12155,7 +12159,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"taskId":"a447c0e34c8245dfaa2758373cf7ec4a","ownerId":"user-1","taskType":"EXPORT","taskName":"学生报表导出-2026春季改","businessKey":"3fb1fb9 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"taskId":"e32cd8971e3343cb8cf979eaf0531e7a","ownerId":"user-1","taskType":"EXPORT","taskName":"学生报表导出-2026春季改","businessKey":"8a9cd8d …</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr"/>
@@ -12188,7 +12192,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"3fb1fb9ad06143c3b014b3445f34c7bf","deleted":true},"traceId":"f5beb3e7b9b34aa88f524de5c7048ec3","timestamp":"2026-08-21T11:03:06.21"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a9cd8db6838443eb747df8151b7c596","deleted":true},"traceId":"45877e64c1114afe99f414d26e8e9453","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timesta …</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr"/>
@@ -12221,7 +12225,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"00f9bce3f4ef4cd688de63163f971870","timestamp":"2026-08-21T11:03:06.455"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"e0896d6b216d4cae962f052781cf468e","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:11.096"}</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr"/>
@@ -12254,7 +12258,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"0d4da69927cc4718b1576c7ce5a6650f","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fileExt":"txt","statu …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"ef21bcd0a71946fa83624e19035b30eb","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fileExt":"txt","statu …</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr"/>
@@ -12287,7 +12291,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"4937e8ee6f3640409fcfb65c9a2a5689","timestamp":"2026-08-21T11:03:06.893"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"246baf30fc4744768a44b3ae4aed73f8","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:11.498"}</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr"/>
@@ -12320,7 +12324,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"上传文件不能为空","data":null,"traceId":"541218480d88486abc6f085a5600b218","timestamp":"2026-08-21T11:03:07.155"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"上传文件不能为空","data":null,"traceId":"1c36835ff4724dcfbf3e7cbbcccf3222","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:11.686"}</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr"/>
@@ -12353,7 +12357,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件内容疑似可执行程序，originalName=evil.xlsx","data":null,"traceId":"46cd4c5be2ae41ca83d502cb45920557","timestamp":"2026-08-21T11:03:07.531"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件内容疑似可执行程序，originalName=evil.xlsx","data":null,"traceId":"a0436f3a1c63429da759aa8706d98bce","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10 …</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -12390,7 +12394,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":true,"file":{"fileId":"0d4da69927cc4718b1576c7ce5a6650f","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":true,"file":{"fileId":"ef21bcd0a71946fa83624e19035b30eb","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d …</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr"/>
@@ -12423,7 +12427,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":false,"file":null},"traceId":"758729c6386a424b876472894e3c1d55","timestamp":"2026-08-21T11:03:08.061"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":false,"file":null},"traceId":"f4a8a0e89d0a4bb59ec1a11571b98b2e","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:12.286"}</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr"/>
@@ -12456,7 +12460,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 不能为空","data":null,"traceId":"5b0c193399dd44be824e20ffaad09e0c","timestamp":"2026-08-21T11:03:08.321"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 不能为空","data":null,"traceId":"7410d934c666402ca50b1dc47a7be49d","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:12.506"}</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr"/>
@@ -12489,7 +12493,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"8afce5ad38ff45439f82b61249b67e68","timestamp":"2026-08-21T11:03:08.537"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"ebb212b294584014b07ef054ef67c257","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:12.7"}</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr"/>
@@ -12522,7 +12526,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件大小必须大于 0","data":null,"traceId":"53da59adbe8d4552b2d206e126f4d060","timestamp":"2026-08-21T11:03:08.743"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件大小必须大于 0","data":null,"traceId":"012112e07ae2497397ebbc18e49414dc","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:12.886"}</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr"/>
@@ -12555,7 +12559,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"0d4da69927cc4718b1576c7ce5a6650f","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fi …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"ef21bcd0a71946fa83624e19035b30eb","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fi …</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr"/>
@@ -12588,7 +12592,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"6d8dfb1960f24e26908fcb2d4f49f2e1","timestamp":"2026-08-21T11:03:09.161"}</t>
+          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"442c7767bc3a4adca518074d69efcf43","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:13.261"}</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr"/>
@@ -12621,7 +12625,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":25,"pageNo":1,"pageSize":5,"records":[{"fileId":"0d4da69927cc4718b1576c7ce5a6650f","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":29,"pageNo":1,"pageSize":5,"records":[{"fileId":"ef21bcd0a71946fa83624e19035b30eb","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223," …</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr"/>
@@ -12683,7 +12687,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"ef2acce117e14cf9aea00b1971b7eb28","timestamp":"2026-08-21T11:03:09.85"}</t>
+          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"5dd11cd68d9e4532b956ed31cd4ad906","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:13.787"}</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr"/>
@@ -12716,7 +12720,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":true,"uploadId":null,"fileId":"0d4da69927cc4718b1576c7ce5a6650f","uploadUrl":null,"objectKey":null,"expireMinutes":null,"file":{"fileId":"0d4da69927cc4718b1576c7ce5a6650 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":true,"uploadId":null,"fileId":"ef21bcd0a71946fa83624e19035b30eb","uploadUrl":null,"objectKey":null,"expireMinutes":null,"file":{"fileId":"ef21bcd0a71946fa83624e19035b30e …</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr"/>
@@ -12749,7 +12753,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"e9343db0b1c6486ebab085c61e9fe3f7","timestamp":"2026-08-21T11:03:10.265"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"e6865842d33a4a148aaff437a5f99164","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:14.086"}</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr"/>
@@ -12782,7 +12786,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"88cde7f247314db09902787ade2bec80","timestamp":"2026-08-21T11:03:10.452"}</t>
+          <t>{"success":false,"code":"FILE_UPLOAD_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"f8b0de18189c489e9f43d761ac151970","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:14.263"}</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr"/>
@@ -12815,7 +12819,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"185665793a26433ab621915d71f9efe2","fileId":"32e4d4e697334041a079f5c290e08234","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"74bca286f20e4d6298e9dab3b74214f2","fileId":"98fce990445c440292b6b0ff5bc62b09","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr"/>
@@ -12848,7 +12852,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"uploadId":"185665793a26433ab621915d71f9efe2","partCount":3,"uploadedParts":[1,2]},"traceId":"56448cdbbbaa48048a143874ba8350b8","timestamp":"2026-08-21T11:04:34.362"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"uploadId":"74bca286f20e4d6298e9dab3b74214f2","partCount":3,"uploadedParts":[1,2]},"traceId":"0f5164f9601242c6a70ed03577f6cbe2","bizId":null,"retryable":null,"suggestion":null,"fi …</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
@@ -12885,7 +12889,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"32e4d4e697334041a079f5c290e08234","ownerId":"user-1","originalName":"big.bin","contentType":null,"fileSize":12582912,"fileMd5":"d4f79b4066eeab2fdd4ffeb11e211d19","fileEx …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"98fce990445c440292b6b0ff5bc62b09","ownerId":"user-1","originalName":"big.bin","contentType":null,"fileSize":12582912,"fileMd5":"fb763671c941dc55e4be690e7e0abcf1","fileEx …</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr"/>
@@ -12918,7 +12922,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"cf2e15d648c749c2a569082bedcb4ac9","timestamp":"2026-08-21T11:04:54.676"}</t>
+          <t>{"success":false,"code":"FILE_UPLOAD_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"9579e455a7134e26894ea900ed04e5e2","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:24.54"}</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr"/>
@@ -12951,7 +12955,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"9e9e2100e2aa4eaebe2486b32c3faf17","fileId":"3548569735114270b676862dd622e0bf","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"5b485043ec7c4f3bbb8685afdc4507f3","fileId":"15feae040eef4c1d80d1fe9f5d89ac63","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr"/>
@@ -12984,7 +12988,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"9e9e2100e2aa4eaebe2486b32c3faf17"},"traceId":"55f29f6eb55d4a52a75c1464fbdcf06e","timestamp":"2026-08-21T11:04:55.731"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"5b485043ec7c4f3bbb8685afdc4507f3"},"traceId":"d39fa309d8b34a5c86dbef31daa9a622","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr"/>
@@ -13017,12 +13021,12 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"9e9e2100e2aa4eaebe2486b32c3faf17"},"traceId":"d26345b164f142899f64aedd88e91aee","timestamp":"2026-08-21T11:04:56.105"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"5b485043ec7c4f3bbb8685afdc4507f3"},"traceId":"0e2b93ee2c6648e9b96f957bb62b688d","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>R19 行为变更：重复 abort 幂等化（200）</t>
+          <t>R19 起重复 abort 幂等（onAborted 回调），返回 200 aborted=true</t>
         </is>
       </c>
     </row>
@@ -13054,7 +13058,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"6d444a64d14040a89a15933d033f06dc","timestamp":"2026-08-21T11:04:56.654"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"1ca7f8ef12104f81b2fa483a100a14a0","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:25.421"}</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr"/>
@@ -13087,7 +13091,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"deleted":true,"fileId":"0d4da69927cc4718b1576c7ce5a6650f"},"traceId":"2ffc3bcc02754502a44bffb7fee42032","timestamp":"2026-08-21T11:04:57.144"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"deleted":true,"fileId":"ef21bcd0a71946fa83624e19035b30eb"},"traceId":"51940cc0baaf4c4a8362f4acd2a5becd","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timest …</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr"/>
@@ -13120,7 +13124,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"a2f17b1b74254d2a82e867b2734d74c1","timestamp":"2026-08-21T11:04:57.387"}</t>
+          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"43c5fc0161ca49bf8d947564e67ff65a","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:25.867"}</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr"/>
@@ -13153,7 +13157,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"文件不存在","data":null,"traceId":"c7bb842f64b944c09dde47bac3a79ecf","timestamp":"2026-08-21T11:04:57.666"}</t>
+          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"4539356785294ca78847339dc1c363b3","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:26.077"}</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr"/>
@@ -13166,7 +13170,7 @@
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>标准环境 R19（执行租约版，2026-08-21）：总 77  ✅PASS 77  ❌FAIL 0 —— task:execution 租约实测捕获；abort 幂等行为变更已同步用例；单测 104/104</t>
+          <t>标准环境 R22（学生查询+游标分页版，2026-08-22 10:15）：总 77  ✅PASS 77  ❌FAIL 0 —— 过滤精确命中/参数 400/游标推进/401 鉴权；分页越界 400 行为变更已同步；单测 138/138</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add compensation auto executor
</commit_message>
<xml_diff>
--- a/docs/test/接口扁平化测试用例.xlsx
+++ b/docs/test/接口扁平化测试用例.xlsx
@@ -9,12 +9,12 @@
   <sheets>
     <sheet name="测试用例" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="接口参数列表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="执行结果(标准环境R22)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="执行结果(标准环境R24)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试用例'!$A$1:$M$136</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'接口参数列表'!$A$1:$K$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'执行结果(标准环境R22)'!$A$1:$G$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'执行结果(标准环境R24)'!$A$1:$G$78</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -10593,7 +10593,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"SECURITY_UNAUTHORIZED","message":"请先登录","data":null,"traceId":"70162071950c448ba1057f12e4582bc4","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:04:57.972"}</t>
+          <t>{"success":false,"code":"SECURITY_UNAUTHORIZED","message":"请先登录","data":null,"traceId":"bba782fd4c454b2eada3a3be1390a1bc","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:11.99"}</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"count":3},"traceId":"1ccc82d3495e4e499904b52982929d84","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:04:58.198"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"count":3},"traceId":"ea356d0bbcbb4072b178821e98b123d1","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:12.36"}</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
@@ -10663,7 +10663,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":3,"count":6,"elapsedMs":7},"traceId":"a5484de817df4d08bc1ad6244bd33298","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:04 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":3,"count":6,"elapsedMs":43},"traceId":"839b0a55c37240bc9e1413dc99a461af","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:0 …</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr"/>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":0,"count":6,"elapsedMs":2},"traceId":"49a97b8292884130a42e8b689a897c6e","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:04 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"inserted":0,"count":6,"elapsedMs":4},"traceId":"d426e1969fb8477e96b0d945140c3500","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08 …</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr"/>
@@ -10729,7 +10729,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"请求参数类型错误","data":null,"traceId":"fe3c86936320497fad9866cf676c7a0a","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:04:58.785"}</t>
+          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"请求参数类型错误","data":null,"traceId":"d9d703b52607447aa65b636fe1e47857","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:13.119"}</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
@@ -10762,12 +10762,12 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>PK�P][Content_Types].xml�S�n�0����*6�PU�C���\{�X�%����]8�R� q�cfgfW�d�q�ZCB|��|�*�*h㻆},^�{Va�^K&lt;4�6�N�XQ�ǆ�9�!P��$��҆�d�c�D�j);��ѝP�g��E�M'O�ʕ����H7L�h���R���G��^�'�{��zސʮB��3�˙��h.�h�W�жF�j娄C …</t>
+          <t>PKY][Content_Types].xml�S�n�0����*6�PU�C���\{�X�%����]8�R� q�cfgfW�d�q�ZCB|��|�*�*h㻆},^�{Va�^K&lt;4�6�N�XQ�ǆ�9�!P��$��҆�d�c�D�j);��ѝP�g��E�M'O�ʕ����H7L�h���R���G��^�'�{��zސʮB��3�˙��h.�h�W�жF�j娄C …</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>模板已下载 3578 字节</t>
+          <t>模板已下载 3577 字节</t>
         </is>
       </c>
     </row>
@@ -10799,7 +10799,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"d1bbb191375d403585ef7690f53db10b","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"c4ffbc6c119444adb35b04fa53d1b334","ownerId":"user-1","status":"CREATED","progressPercent":0,"totalCount":0,"completedCount":0,"retryCount":0,"maxRetryCount":3,"errorMess …</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr"/>
@@ -10832,7 +10832,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"d1bbb191375d403585ef7690f53db10b","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"totalCount":3,"completedCount":3,"retryCount":0,"maxRetryCount":3,"errorMe …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"c4ffbc6c119444adb35b04fa53d1b334","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"totalCount":3,"completedCount":3,"retryCount":0,"maxRetryCount":3,"errorMe …</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -10869,7 +10869,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"EXCEL_TASK_NOT_FOUND","message":"导入任务不存在","data":null,"traceId":"ddd17c435ee54347927a86ea60ce6628","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:01.998"}</t>
+          <t>{"success":false,"code":"EXCEL_TASK_NOT_FOUND","message":"导入任务不存在","data":null,"traceId":"c9a26aace705472a896321e40dbaaf7a","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:17.916"}</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr"/>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"EXCEL_FILE_NOT_FOUND","message":"导入错误明细文件不存在","data":null,"traceId":"e53941234d7d44efbdcd7502e4e58ca0","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:02.246"}</t>
+          <t>{"success":false,"code":"EXCEL_FILE_NOT_FOUND","message":"导入错误明细文件不存在","data":null,"traceId":"b7b69903cb0d460ab2d00cf11a88c73e","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:18.154"}</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
@@ -10935,7 +10935,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"b7bc32e656ef43cca8502f8308cdd668","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:02.469"}</t>
+          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"3c173dfeb0214069938a9ea2bd4171d6","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:18.352"}</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr"/>
@@ -10968,7 +10968,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"导入文件不能为空","data":null,"traceId":"cf61812007ae415c876a923beab8c9d1","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:02.681"}</t>
+          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"导入文件不能为空","data":null,"traceId":"a4b8c69e5eaf4f1b9c402b9e4a130ed9","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:18.617"}</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr"/>
@@ -11001,7 +11001,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"导入文件格式错误，请上传 .xlsx 文件","data":null,"traceId":"2dea2f57f7db49e9b19a6f5fc06ff546","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:02.844"}</t>
+          <t>{"success":false,"code":"EXCEL_PARAM_ERROR","message":"导入文件格式错误，请上传 .xlsx 文件","data":null,"traceId":"5139d232db3f4eee9e88a6caad030b1f","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:18.832"}</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -11038,7 +11038,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"438d4fb5be7444deae77bf58a3100af8","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr"/>
@@ -11071,7 +11071,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"92345433cb134e98b86e527d034421e2","canceled":false},"traceId":"1566d9e58a494366b2f0110f4da5c98c","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"07aa2771add54c2082432ebf49f8b50f","canceled":false},"traceId":"9b8f04791ee949dda27c311332aebf99","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr"/>
@@ -11104,7 +11104,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"total":3,"exported":3,"sheetCount":1,"retryCount":0,"maxRetryCount":3,"fil …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"438d4fb5be7444deae77bf58a3100af8","ownerId":"user-1","status":"SUCCESS","progressPercent":100,"total":3,"exported":3,"sheetCount":1,"retryCount":0,"maxRetryCount":3,"fil …</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -11141,7 +11141,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>{"timestamp":"2026-08-22T02:05:03.870+00:00","status":404,"error":"Not Found","path":"/api/excel/not-exist"}</t>
+          <t>{"timestamp":"2026-08-22T03:08:20.004+00:00","status":404,"error":"Not Found","path":"/api/excel/not-exist"}</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr"/>
@@ -11174,7 +11174,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"EXCEL_TASK_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"7f86aa0e808d47b3b0fbf99da0f4253a","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:04.067"}</t>
+          <t>{"success":false,"code":"EXCEL_TASK_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"34a5e73c018a4289aabc6d3b8d4bcc3f","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:20.192"}</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr"/>
@@ -11240,7 +11240,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"EXCEL_TASK_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"b2505d41ca3b4784bd827625fd7270c7","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:04.438"}</t>
+          <t>{"success":false,"code":"EXCEL_TASK_NOT_FOUND","message":"导出任务不存在","data":null,"traceId":"a6986cf7c29a4e4bb3b644be8af44654","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:20.657"}</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
@@ -11273,7 +11273,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":122,"pageNo":1,"pageSize":5,"records":[{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"b7ff83e8167a4 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":128,"pageNo":1,"pageSize":5,"records":[{"taskId":"438d4fb5be7444deae77bf58a3100af8","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"ce4f0d473bf94 …</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
@@ -11306,7 +11306,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":122,"pageNo":1,"pageSize":20,"records":[{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"b7ff83e8167a …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":128,"pageNo":1,"pageSize":20,"records":[{"taskId":"438d4fb5be7444deae77bf58a3100af8","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"ce4f0d473bf9 …</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr"/>
@@ -11339,12 +11339,12 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"TASK_PARAM_ERROR","message":"请求参数校验失败","data":null,"traceId":"2efab826a1fb4b349442d09a32ee336c","bizId":null,"retryable":false,"suggestion":"请根据 fieldErrors 修正请求参数","fieldErrors":[{"field":"pageSize","message":"每页条数 …</t>
+          <t>{"success":false,"code":"TASK_PARAM_ERROR","message":"请求参数校验失败","data":null,"traceId":"7d97bea4692044c29f18534f53fa0926","bizId":null,"retryable":false,"suggestion":"请根据 fieldErrors 修正请求参数","fieldErrors":[{"field":"pageNo","message":"页码必须大于 …</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>R22 行为变更：越界分页参数 400 拒绝（ERR-03 Bean Validation）</t>
+          <t>R22 起越界分页参数由静默钳制改为 Bean Validation 400 拒绝（ERR-03）</t>
         </is>
       </c>
     </row>
@@ -11376,7 +11376,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"TASK_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskStatus.GARBAGE","data":null,"traceId":"c2d53040642747b79a9631d263c73b04","bizId":null,"retryable":null,"suggestion":null,"field …</t>
+          <t>{"success":false,"code":"TASK_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskStatus.GARBAGE","data":null,"traceId":"41b6e36ae72d4e0f9bc9ec02561fa192","bizId":null,"retryable":null,"suggestion":null,"field …</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -11413,7 +11413,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"TASK_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskType.GARBAGE","data":null,"traceId":"21234cfefbc5416d95412d22bcd4aa14","bizId":null,"retryable":null,"suggestion":null,"fieldEr …</t>
+          <t>{"success":false,"code":"TASK_PARAM_ERROR","message":"No enum constant com.huang.demo.task.domain.model.AsyncTaskType.GARBAGE","data":null,"traceId":"e9bb3b8451b7439cbef910b793a923de","bizId":null,"retryable":null,"suggestion":null,"fieldEr …</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -11450,7 +11450,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"b7ff83e8167a47b9a7989d218c2aee5d","status":"SUCCESS","progres …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"438d4fb5be7444deae77bf58a3100af8","ownerId":"user-1","taskType":"EXPORT","taskName":"学生数据导出","businessKey":"ce4f0d473bf947be8ce82593d517a3e1","status":"SUCCESS","progres …</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr"/>
@@ -11483,7 +11483,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"TASK_NOT_FOUND","message":"任务不存在","data":null,"traceId":"c4001e13accb4ca497f1ead62eb0722e","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:06.188"}</t>
+          <t>{"success":false,"code":"TASK_NOT_FOUND","message":"任务不存在","data":null,"traceId":"117138b6d5be4f03a251d4d84b6d8632","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:22.658"}</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
@@ -11516,7 +11516,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"TASK_NOT_FOUND","message":"任务不存在","data":null,"traceId":"5f69a0162109454e919d5856ab7c5fe3","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:06.381"}</t>
+          <t>{"success":false,"code":"TASK_NOT_FOUND","message":"任务不存在","data":null,"traceId":"4b6497da7d5c448594f9edb739257702","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:22.899"}</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr"/>
@@ -11549,7 +11549,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"ce54b1ef1b2d46c0931dcbf01b60c445","canceled":false},"traceId":"010d78d324934cc294347d8a23412936","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"438d4fb5be7444deae77bf58a3100af8","canceled":false},"traceId":"906163c5da3344a3828ff7cf2a568936","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"TASK_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"fe9d046fdf3b49a8885f30145b3288e3","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:0 …</t>
+          <t>{"success":false,"code":"TASK_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"999324b37a3643cdad49b6744c5e245c","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:2 …</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"TASK_NOT_FOUND","message":"任务不存在","data":null,"traceId":"89985f5a6b1149399a0a251695eafc7b","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:07.184"}</t>
+          <t>{"success":false,"code":"TASK_NOT_FOUND","message":"任务不存在","data":null,"traceId":"89a0629829bd4b0dab7c991b6d7540aa","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:23.639"}</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr"/>
@@ -11656,7 +11656,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"TASK_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"3f0e8fb2a47f40f58f9d82dda8ef8c48","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:0 …</t>
+          <t>{"success":false,"code":"TASK_STATE_CONFLICT","message":"当前任务状态不允许重试，status=SUCCESS","data":null,"traceId":"992f84e9b95b438b88651a5e326d16ea","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:2 …</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -11693,7 +11693,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a9cd8db6838443eb747df8151b7c596","ownerId":"user-1","runControlCode":"RT87364303","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a940c1d9d3141a1a4ec343b57bac6b6","ownerId":"user-1","runControlCode":"RT87368104","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr"/>
@@ -11726,7 +11726,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码不能为空","data":null,"traceId":"783c68fa85724761b3e4d55d3078bc17","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:08.076"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码不能为空","data":null,"traceId":"7ccaf73ae7844110b52045a656c079e1","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:24.584"}</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr"/>
@@ -11759,7 +11759,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码已存在","data":null,"traceId":"51809234343b48d6853d37d82f2d61f2","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:08.257"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"运行控制编码已存在","data":null,"traceId":"0974b501da8d4d5eae25890f3b39061a","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:24.87"}</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr"/>
@@ -11792,7 +11792,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄必须在0到150之间","data":null,"traceId":"33b30b25f95748f5b3da9bc850c27f10","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:08.456"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄必须在0到150之间","data":null,"traceId":"e53d0bfc23e14604afd13fc9b5b76ccb","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:25.083"}</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr"/>
@@ -11825,7 +11825,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最大年龄必须在0到150之间","data":null,"traceId":"8936f866a34943f4a5baabd453252adf","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:08.684"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最大年龄必须在0到150之间","data":null,"traceId":"a9ec2c0931f9455ba078d26bef726447","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:25.264"}</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
@@ -11858,7 +11858,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"d61401405c1d4b09baffaf0bd21deea6","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:08.867"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"6122237b4cf8424286e885b29a6e916b","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:25.486"}</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr"/>
@@ -11891,7 +11891,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"runId":"8a9cd8db6838443eb747df8151b7c596","ownerId":"user-1","runControlCode":"RT87364303","runName":"2026春季测试","studentNo":"T202608 …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"runId":"8a940c1d9d3141a1a4ec343b57bac6b6","ownerId":"user-1","runControlCode":"RT87368104","runName":"2026春季测试","studentNo":"T202608 …</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr"/>
@@ -11924,7 +11924,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.excel.domain.model.StudentReportRunStatus.GARBAGE","data":null,"traceId":"0340bae5d8354fe5bf2b5075dadc9075","bizId":null,"retryable":null,"suggestion":n …</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"No enum constant com.huang.demo.excel.domain.model.StudentReportRunStatus.GARBAGE","data":null,"traceId":"df5a473fdd124e308ebc9d8ef16305d5","bizId":null,"retryable":null,"suggestion":n …</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
@@ -11961,7 +11961,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a9cd8db6838443eb747df8151b7c596","ownerId":"user-1","runControlCode":"RT87364303","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a940c1d9d3141a1a4ec343b57bac6b6","ownerId":"user-1","runControlCode":"RT87368104","runName":"2026春季测试","studentNo":"T20260814001","nameKeyword":null,"className":null,"ge …</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
@@ -11994,7 +11994,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"cd426004567f4067b9f19c4be3916762","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:09.672"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"afce64fae71846faaba111e0c8d8084a","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:26.438"}</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr"/>
@@ -12027,7 +12027,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"dc2aadce2dec44a8b9f1320232f76e85","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:09.882"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"93747ddc76894d308d8815cfd3583d86","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:26.713"}</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr"/>
@@ -12060,7 +12060,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a9cd8db6838443eb747df8151b7c596","ownerId":"user-1","runControlCode":"RT87364303","runName":"2026春季改","studentNo":null,"nameKeyword":null,"className":"一班","gender":null, …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a940c1d9d3141a1a4ec343b57bac6b6","ownerId":"user-1","runControlCode":"RT87368104","runName":"2026春季改","studentNo":null,"nameKeyword":null,"className":"一班","gender":null, …</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr"/>
@@ -12093,7 +12093,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"58a9f298a7dd4203b11ea8f55b4ab7a7","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:10.299"}</t>
+          <t>{"success":false,"code":"COMMON_PARAM_ERROR","message":"最小年龄不能大于最大年龄","data":null,"traceId":"55e47fc45250453e912b6898c7aed9ce","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:27.146"}</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr"/>
@@ -12126,7 +12126,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"e32cd8971e3343cb8cf979eaf0531e7a","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"taskId":"18aaf20c3b2c43a8949a9a495a3bc174","ownerId":"user-1","status":"QUEUED","progressPercent":0,"total":0,"exported":0,"sheetCount":0,"retryCount":0,"maxRetryCount":3,"fileNa …</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr"/>
@@ -12159,7 +12159,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"taskId":"e32cd8971e3343cb8cf979eaf0531e7a","ownerId":"user-1","taskType":"EXPORT","taskName":"学生报表导出-2026春季改","businessKey":"8a9cd8d …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":1,"pageNo":1,"pageSize":5,"records":[{"taskId":"18aaf20c3b2c43a8949a9a495a3bc174","ownerId":"user-1","taskType":"EXPORT","taskName":"学生报表导出-2026春季改","businessKey":"8a940c1 …</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr"/>
@@ -12192,7 +12192,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a9cd8db6838443eb747df8151b7c596","deleted":true},"traceId":"45877e64c1114afe99f414d26e8e9453","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timesta …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"runId":"8a940c1d9d3141a1a4ec343b57bac6b6","deleted":true},"traceId":"da9ea0e07e454043ace45a1acc0d2309","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timesta …</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr"/>
@@ -12225,7 +12225,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"e0896d6b216d4cae962f052781cf468e","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:11.096"}</t>
+          <t>{"success":false,"code":"COMMON_NOT_FOUND","message":"运行控制不存在","data":null,"traceId":"2db2e878d2544a508a15e7aa91c5345d","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:28.044"}</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr"/>
@@ -12258,7 +12258,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"ef21bcd0a71946fa83624e19035b30eb","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fileExt":"txt","statu …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"4e12dafbf3854bb4885cbf5796a54a52","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fileExt":"txt","statu …</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr"/>
@@ -12291,7 +12291,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"246baf30fc4744768a44b3ae4aed73f8","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:11.498"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"请求 Content-Type 不支持","data":null,"traceId":"880863a5d550494eb36ed400ccc61305","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:28.74"}</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr"/>
@@ -12324,7 +12324,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"上传文件不能为空","data":null,"traceId":"1c36835ff4724dcfbf3e7cbbcccf3222","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:11.686"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"上传文件不能为空","data":null,"traceId":"bf633fd246694ba89271f1303faf1169","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:29.026"}</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr"/>
@@ -12357,7 +12357,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件内容疑似可执行程序，originalName=evil.xlsx","data":null,"traceId":"a0436f3a1c63429da759aa8706d98bce","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10 …</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件内容疑似可执行程序，originalName=evil.xlsx","data":null,"traceId":"43e3cd1d7f8f4a13ac5699a938a3cffa","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11 …</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -12394,7 +12394,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":true,"file":{"fileId":"ef21bcd0a71946fa83624e19035b30eb","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":true,"file":{"fileId":"4e12dafbf3854bb4885cbf5796a54a52","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d …</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr"/>
@@ -12427,7 +12427,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":false,"file":null},"traceId":"f4a8a0e89d0a4bb59ec1a11571b98b2e","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:12.286"}</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"exists":false,"file":null},"traceId":"bee53f1dbe8e4e5bbcad147d1c5ec3c6","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:29.679"}</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr"/>
@@ -12460,7 +12460,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 不能为空","data":null,"traceId":"7410d934c666402ca50b1dc47a7be49d","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:12.506"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 不能为空","data":null,"traceId":"5536f684391f4b328d6eb291f04e9878","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:29.861"}</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr"/>
@@ -12493,7 +12493,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"ebb212b294584014b07ef054ef67c257","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:12.7"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"2b7ca9624ae94a35ae459c8c0aa0411b","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:30.113"}</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr"/>
@@ -12526,7 +12526,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件大小必须大于 0","data":null,"traceId":"012112e07ae2497397ebbc18e49414dc","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:12.886"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件大小必须大于 0","data":null,"traceId":"8daa7ab5a9b54f35a0bda663d8df5501","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:30.432"}</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr"/>
@@ -12559,7 +12559,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"ef21bcd0a71946fa83624e19035b30eb","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fi …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"4e12dafbf3854bb4885cbf5796a54a52","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223,"fileMd5":"62de957351c4d5d84f32b1f6c9d284a6","fi …</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr"/>
@@ -12592,7 +12592,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"442c7767bc3a4adca518074d69efcf43","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:13.261"}</t>
+          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"fd341183489d4deab7d8f6c22228ba99","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:31.044"}</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr"/>
@@ -12625,7 +12625,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":29,"pageNo":1,"pageSize":5,"records":[{"fileId":"ef21bcd0a71946fa83624e19035b30eb","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"total":31,"pageNo":1,"pageSize":5,"records":[{"fileId":"4e12dafbf3854bb4885cbf5796a54a52","ownerId":"user-1","originalName":"demo.txt","contentType":"text/plain","fileSize":223," …</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr"/>
@@ -12687,7 +12687,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"5dd11cd68d9e4532b956ed31cd4ad906","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:13.787"}</t>
+          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"ff9932ad94844d45acfafa760a41636e","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:32.017"}</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr"/>
@@ -12720,7 +12720,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":true,"uploadId":null,"fileId":"ef21bcd0a71946fa83624e19035b30eb","uploadUrl":null,"objectKey":null,"expireMinutes":null,"file":{"fileId":"ef21bcd0a71946fa83624e19035b30e …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":true,"uploadId":null,"fileId":"4e12dafbf3854bb4885cbf5796a54a52","uploadUrl":null,"objectKey":null,"expireMinutes":null,"file":{"fileId":"4e12dafbf3854bb4885cbf5796a54a5 …</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr"/>
@@ -12753,7 +12753,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"e6865842d33a4a148aaff437a5f99164","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:14.086"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"45046cf1598e4709b23e77b1c4345249","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:32.643"}</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr"/>
@@ -12786,7 +12786,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_UPLOAD_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"f8b0de18189c489e9f43d761ac151970","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:14.263"}</t>
+          <t>{"success":false,"code":"FILE_UPLOAD_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"fb368915343b429e8fca3635dca463ab","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:32.909"}</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr"/>
@@ -12819,7 +12819,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"74bca286f20e4d6298e9dab3b74214f2","fileId":"98fce990445c440292b6b0ff5bc62b09","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"5e092492cf4343d2b344d26f3bfc4b93","fileId":"50d01644a53e417c86dad58af7241795","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr"/>
@@ -12852,7 +12852,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"uploadId":"74bca286f20e4d6298e9dab3b74214f2","partCount":3,"uploadedParts":[1,2]},"traceId":"0f5164f9601242c6a70ed03577f6cbe2","bizId":null,"retryable":null,"suggestion":null,"fi …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"uploadId":"5e092492cf4343d2b344d26f3bfc4b93","partCount":3,"uploadedParts":[1,2]},"traceId":"402bdc4e4a2a4b90a9d796b9814e2660","bizId":null,"retryable":null,"suggestion":null,"fi …</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
@@ -12889,7 +12889,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"98fce990445c440292b6b0ff5bc62b09","ownerId":"user-1","originalName":"big.bin","contentType":null,"fileSize":12582912,"fileMd5":"fb763671c941dc55e4be690e7e0abcf1","fileEx …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"fileId":"50d01644a53e417c86dad58af7241795","ownerId":"user-1","originalName":"big.bin","contentType":null,"fileSize":12582912,"fileMd5":"75e9b41a8b5db7fb3934241afc8fcec9","fileEx …</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr"/>
@@ -12922,7 +12922,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_UPLOAD_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"9579e455a7134e26894ea900ed04e5e2","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:24.54"}</t>
+          <t>{"success":false,"code":"FILE_UPLOAD_NOT_FOUND","message":"上传任务不存在","data":null,"traceId":"1fbb14d69bef405eba5a6b2aa0cb2b34","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:45.463"}</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr"/>
@@ -12955,7 +12955,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"5b485043ec7c4f3bbb8685afdc4507f3","fileId":"15feae040eef4c1d80d1fe9f5d89ac63","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"instant":false,"uploadId":"8de1734ba1dc41e5ba2f68836ad2391d","fileId":"89ecc7bf51784403985356a6afdf795e","fileSize":12582912,"partSize":5242880,"partCount":3,"expireMinutes":30," …</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr"/>
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"5b485043ec7c4f3bbb8685afdc4507f3"},"traceId":"d39fa309d8b34a5c86dbef31daa9a622","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"8de1734ba1dc41e5ba2f68836ad2391d"},"traceId":"003d9be59a8b4686bf742609ae8f5dfc","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr"/>
@@ -13021,7 +13021,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"5b485043ec7c4f3bbb8685afdc4507f3"},"traceId":"0e2b93ee2c6648e9b96f957bb62b688d","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"aborted":true,"uploadId":"8de1734ba1dc41e5ba2f68836ad2391d"},"traceId":"aad6250f9e764357932d7fedc387cbfe","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"time …</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
@@ -13058,7 +13058,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"1ca7f8ef12104f81b2fa483a100a14a0","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:25.421"}</t>
+          <t>{"success":false,"code":"FILE_PARAM_ERROR","message":"文件 MD5 格式不正确","data":null,"traceId":"68eac9345d1d4ce4b9ffea70d22bb568","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:46.438"}</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr"/>
@@ -13091,7 +13091,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"deleted":true,"fileId":"ef21bcd0a71946fa83624e19035b30eb"},"traceId":"51940cc0baaf4c4a8362f4acd2a5becd","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timest …</t>
+          <t>{"success":true,"code":"SUCCESS","message":"success","data":{"deleted":true,"fileId":"4e12dafbf3854bb4885cbf5796a54a52"},"traceId":"4957767b6e7043d59a586a1748a64adb","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timest …</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr"/>
@@ -13124,7 +13124,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"43c5fc0161ca49bf8d947564e67ff65a","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:25.867"}</t>
+          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"df4699cc52214bb7a3b56992e358d1ec","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:46.902"}</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr"/>
@@ -13157,7 +13157,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"4539356785294ca78847339dc1c363b3","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T10:05:26.077"}</t>
+          <t>{"success":false,"code":"FILE_NOT_FOUND","message":"文件不存在","data":null,"traceId":"addf5b39d0e04f1fb5263d74e88f25c9","bizId":null,"retryable":null,"suggestion":null,"fieldErrors":null,"timestamp":"2026-08-22T11:08:47.118"}</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr"/>
@@ -13170,7 +13170,7 @@
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
-          <t>标准环境 R22（学生查询+游标分页版，2026-08-22 10:15）：总 77  ✅PASS 77  ❌FAIL 0 —— 过滤精确命中/参数 400/游标推进/401 鉴权；分页越界 400 行为变更已同步；单测 138/138</t>
+          <t>标准环境 R24（自动补偿执行器版，2026-08-22 11:10）：总 77  ✅PASS 77  ❌FAIL 0 —— 43 条真实补偿记录自动重放（孤儿清理 SUCCESS×5、不可恢复类型退避/人工分流）；单测 164/164</t>
         </is>
       </c>
     </row>

</xml_diff>